<commit_message>
upated location of files
</commit_message>
<xml_diff>
--- a/silver_layer_data_validation_databrick_catalog/queries/validation_queries.xlsx
+++ b/silver_layer_data_validation_databrick_catalog/queries/validation_queries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6800" activeTab="2"/>
+    <workbookView windowWidth="19200" windowHeight="6080" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="db" sheetId="3" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="120">
   <si>
     <t>db_name</t>
   </si>
@@ -150,190 +150,100 @@
     <t>amendment_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\amendment_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\amendment_base.sql</t>
   </si>
   <si>
     <t>application_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\application_base.sql</t>
-  </si>
-  <si>
     <t>application_support_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\application_support_base.sql</t>
-  </si>
-  <si>
     <t>assessment_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\assessment_base.sql</t>
-  </si>
-  <si>
     <t>certification_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\certification_base.sql</t>
-  </si>
-  <si>
     <t>customer_enterprise_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\customer_enterprise_base.sql</t>
-  </si>
-  <si>
     <t>customer_individual_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\ticket_base.sql</t>
-  </si>
-  <si>
     <t>employee_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\employee_base.sql</t>
-  </si>
-  <si>
     <t>financing_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\financing_base.sql</t>
-  </si>
-  <si>
     <t>iban_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\iban_base.sql</t>
-  </si>
-  <si>
     <t>moic_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\moic_base.sql</t>
-  </si>
-  <si>
     <t>payment_assessment_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\payment_assessment_base.sql</t>
-  </si>
-  <si>
     <t>payment_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\payment_base.sql</t>
-  </si>
-  <si>
     <t>payment_plan_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\payment_plan_base.sql</t>
-  </si>
-  <si>
     <t>payment_support_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\payment_support_base.sql</t>
-  </si>
-  <si>
     <t>product_services_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\product_services_base.sql</t>
-  </si>
-  <si>
     <t>program_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\program_base.sql</t>
-  </si>
-  <si>
     <t>sector_isic_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\sector_isic_base.sql</t>
-  </si>
-  <si>
     <t>security_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\security_base.sql</t>
-  </si>
-  <si>
     <t>service_fee_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\service_fee_base.sql</t>
-  </si>
-  <si>
     <t>special_condition_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\special_condition_base.sql</t>
-  </si>
-  <si>
     <t>support_structure_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\support_structure_base.sql</t>
-  </si>
-  <si>
     <t>ticket_base</t>
   </si>
   <si>
     <t>training_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\training_base.sql</t>
-  </si>
-  <si>
     <t>unstructured_questions_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\unstructured_questions_base.sql</t>
-  </si>
-  <si>
     <t>user_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\user_base.sql</t>
-  </si>
-  <si>
     <t>wage_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\wage_base.sql</t>
-  </si>
-  <si>
     <t>workflow_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\workflow_base.sql</t>
-  </si>
-  <si>
     <t>withdrawal_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\withdrawal_base.sql</t>
-  </si>
-  <si>
     <t>infor_dimension_mapping_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\infor\infor_special_project_compare_bronze_silver.sql</t>
-  </si>
-  <si>
     <t>odoo_calender_event_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\odoo\odoo_calender_compare_bronze_silver.sql</t>
-  </si>
-  <si>
     <t>odoo_contact_base</t>
-  </si>
-  <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\jenkins_project\silver_layer_data_validation\queries\sql_union_all_sources\odoo\odoo_contact_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>offline_sheets_dapm_master_sheet</t>
@@ -2051,14 +1961,12 @@
         <v>2</v>
       </c>
       <c r="B3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D3" s="12" t="s">
-        <v>40</v>
-      </c>
+      <c r="D3" s="12"/>
       <c r="E3" s="5"/>
     </row>
     <row r="4" ht="33" customHeight="1" spans="1:5">
@@ -2066,14 +1974,12 @@
         <v>3</v>
       </c>
       <c r="B4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>42</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="D4" s="12"/>
       <c r="E4" s="5"/>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:5">
@@ -2081,14 +1987,12 @@
         <v>4</v>
       </c>
       <c r="B5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>44</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="D5" s="12"/>
       <c r="E5" s="5"/>
     </row>
     <row r="6" ht="33" customHeight="1" spans="1:5">
@@ -2096,14 +2000,12 @@
         <v>5</v>
       </c>
       <c r="B6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>46</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D6" s="12"/>
       <c r="E6" s="5"/>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:5">
@@ -2111,14 +2013,12 @@
         <v>6</v>
       </c>
       <c r="B7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>48</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="D7" s="12"/>
       <c r="E7" s="5"/>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:5">
@@ -2126,14 +2026,12 @@
         <v>7</v>
       </c>
       <c r="B8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>50</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="D8" s="12"/>
       <c r="E8" s="5"/>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:5">
@@ -2141,14 +2039,12 @@
         <v>8</v>
       </c>
       <c r="B9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>52</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="D9" s="12"/>
       <c r="E9" s="5"/>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:5">
@@ -2156,14 +2052,12 @@
         <v>9</v>
       </c>
       <c r="B10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>54</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="D10" s="12"/>
       <c r="E10" s="5"/>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:5">
@@ -2171,14 +2065,12 @@
         <v>10</v>
       </c>
       <c r="B11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>56</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="D11" s="12"/>
       <c r="E11" s="5"/>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:5">
@@ -2186,14 +2078,12 @@
         <v>11</v>
       </c>
       <c r="B12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>58</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="D12" s="12"/>
       <c r="E12" s="5"/>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:5">
@@ -2201,14 +2091,12 @@
         <v>12</v>
       </c>
       <c r="B13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>60</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="D13" s="12"/>
       <c r="E13" s="5"/>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:5">
@@ -2216,14 +2104,12 @@
         <v>13</v>
       </c>
       <c r="B14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>62</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="D14" s="12"/>
       <c r="E14" s="5"/>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:5">
@@ -2231,14 +2117,12 @@
         <v>14</v>
       </c>
       <c r="B15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>64</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="D15" s="12"/>
       <c r="E15" s="5"/>
     </row>
     <row r="16" ht="32" customHeight="1" spans="1:5">
@@ -2246,14 +2130,12 @@
         <v>15</v>
       </c>
       <c r="B16" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>66</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="D16" s="12"/>
       <c r="E16" s="5"/>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:5">
@@ -2261,14 +2143,12 @@
         <v>16</v>
       </c>
       <c r="B17" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>68</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="D17" s="12"/>
       <c r="E17" s="5"/>
     </row>
     <row r="18" customFormat="1" ht="30" customHeight="1" spans="1:5">
@@ -2276,14 +2156,12 @@
         <v>17</v>
       </c>
       <c r="B18" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>70</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="D18" s="12"/>
       <c r="E18" s="5"/>
     </row>
     <row r="19" customFormat="1" ht="30" customHeight="1" spans="1:5">
@@ -2291,14 +2169,12 @@
         <v>18</v>
       </c>
       <c r="B19" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>72</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="D19" s="12"/>
       <c r="E19" s="5"/>
     </row>
     <row r="20" customFormat="1" ht="30" customHeight="1" spans="1:5">
@@ -2306,14 +2182,12 @@
         <v>19</v>
       </c>
       <c r="B20" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>74</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="D20" s="12"/>
       <c r="E20" s="5"/>
     </row>
     <row r="21" customFormat="1" ht="30" customHeight="1" spans="1:5">
@@ -2321,14 +2195,12 @@
         <v>20</v>
       </c>
       <c r="B21" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>76</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="D21" s="12"/>
       <c r="E21" s="5"/>
     </row>
     <row r="22" customFormat="1" ht="30" customHeight="1" spans="1:5">
@@ -2336,14 +2208,12 @@
         <v>21</v>
       </c>
       <c r="B22" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>78</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="D22" s="12"/>
       <c r="E22" s="12"/>
     </row>
     <row r="23" customFormat="1" ht="30" customHeight="1" spans="1:5">
@@ -2351,44 +2221,38 @@
         <v>22</v>
       </c>
       <c r="B23" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="D23" s="12" t="s">
-        <v>80</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="D23" s="12"/>
       <c r="E23" s="5"/>
     </row>
-    <row r="24" s="11" customFormat="1" ht="29" spans="1:5">
+    <row r="24" s="11" customFormat="1" spans="1:5">
       <c r="A24" s="5">
         <v>23</v>
       </c>
       <c r="B24" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>50</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="D24" s="12"/>
       <c r="E24" s="6"/>
     </row>
-    <row r="25" s="11" customFormat="1" ht="29" spans="1:5">
+    <row r="25" s="11" customFormat="1" spans="1:5">
       <c r="A25" s="5">
         <v>24</v>
       </c>
       <c r="B25" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>83</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="D25" s="12"/>
       <c r="E25" s="6"/>
     </row>
     <row r="26" ht="27" customHeight="1" spans="1:5">
@@ -2396,14 +2260,12 @@
         <v>25</v>
       </c>
       <c r="B26" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>85</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="D26" s="12"/>
       <c r="E26" s="5"/>
     </row>
     <row r="27" ht="35" customHeight="1" spans="1:5">
@@ -2411,14 +2273,12 @@
         <v>26</v>
       </c>
       <c r="B27" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>87</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="D27" s="12"/>
       <c r="E27" s="5"/>
     </row>
     <row r="28" ht="35" customHeight="1" spans="1:5">
@@ -2426,14 +2286,12 @@
         <v>27</v>
       </c>
       <c r="B28" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>89</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="D28" s="12"/>
       <c r="E28" s="5"/>
     </row>
     <row r="29" ht="35" customHeight="1" spans="1:5">
@@ -2441,29 +2299,25 @@
         <v>28</v>
       </c>
       <c r="B29" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="D29" s="12" t="s">
-        <v>91</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="D29" s="12"/>
       <c r="E29" s="5"/>
     </row>
-    <row r="30" ht="29" spans="1:5">
+    <row r="30" spans="1:5">
       <c r="A30" s="5">
         <v>29</v>
       </c>
       <c r="B30" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>93</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="D30" s="12"/>
       <c r="E30" s="5"/>
     </row>
     <row r="31" s="11" customFormat="1" ht="32" customHeight="1" spans="1:5">
@@ -2471,14 +2325,12 @@
         <v>30</v>
       </c>
       <c r="B31" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>95</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="D31" s="14"/>
       <c r="E31" s="6"/>
     </row>
     <row r="32" s="11" customFormat="1" ht="29" customHeight="1" spans="1:5">
@@ -2486,14 +2338,12 @@
         <v>31</v>
       </c>
       <c r="B32" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="D32" s="16" t="s">
-        <v>97</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="D32" s="16"/>
       <c r="E32" s="6"/>
     </row>
     <row r="33" s="11" customFormat="1" ht="30" customHeight="1" spans="1:5">
@@ -2501,14 +2351,12 @@
         <v>32</v>
       </c>
       <c r="B33" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="D33" s="16" t="s">
-        <v>99</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="D33" s="16"/>
       <c r="E33" s="6"/>
     </row>
     <row r="34" s="11" customFormat="1" ht="30" customHeight="1" spans="1:5">
@@ -2517,7 +2365,7 @@
         <v>0</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="D34" s="16"/>
       <c r="E34" s="6"/>
@@ -2528,7 +2376,7 @@
         <v>0</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="D35" s="16"/>
       <c r="E35" s="6"/>
@@ -2539,7 +2387,7 @@
         <v>0</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
       <c r="D36" s="16"/>
       <c r="E36" s="6"/>
@@ -2548,7 +2396,7 @@
       <c r="A37" s="6"/>
       <c r="B37" s="6"/>
       <c r="C37" s="15" t="s">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="D37" s="16"/>
       <c r="E37" s="6"/>
@@ -2557,7 +2405,7 @@
       <c r="A38" s="6"/>
       <c r="B38" s="6"/>
       <c r="C38" s="15" t="s">
-        <v>104</v>
+        <v>74</v>
       </c>
       <c r="D38" s="16"/>
       <c r="E38" s="6"/>
@@ -2566,7 +2414,7 @@
       <c r="A39" s="6"/>
       <c r="B39" s="6"/>
       <c r="C39" s="15" t="s">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="D39" s="16"/>
       <c r="E39" s="6"/>
@@ -2575,7 +2423,7 @@
       <c r="A40" s="6"/>
       <c r="B40" s="6"/>
       <c r="C40" s="15" t="s">
-        <v>106</v>
+        <v>76</v>
       </c>
       <c r="D40" s="16"/>
       <c r="E40" s="6"/>
@@ -2584,7 +2432,7 @@
       <c r="A41" s="6"/>
       <c r="B41" s="6"/>
       <c r="C41" s="15" t="s">
-        <v>107</v>
+        <v>77</v>
       </c>
       <c r="D41" s="16"/>
       <c r="E41" s="6"/>
@@ -2593,7 +2441,7 @@
       <c r="A42" s="6"/>
       <c r="B42" s="6"/>
       <c r="C42" s="15" t="s">
-        <v>108</v>
+        <v>78</v>
       </c>
       <c r="D42" s="16"/>
       <c r="E42" s="6"/>
@@ -2602,7 +2450,7 @@
       <c r="A43" s="6"/>
       <c r="B43" s="6"/>
       <c r="C43" s="15" t="s">
-        <v>109</v>
+        <v>79</v>
       </c>
       <c r="D43" s="16"/>
       <c r="E43" s="6"/>
@@ -2611,7 +2459,7 @@
       <c r="A44" s="6"/>
       <c r="B44" s="6"/>
       <c r="C44" s="15" t="s">
-        <v>110</v>
+        <v>80</v>
       </c>
       <c r="D44" s="16"/>
       <c r="E44" s="6"/>
@@ -3218,13 +3066,13 @@
         <v>34</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>111</v>
+        <v>81</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -3239,7 +3087,7 @@
       </c>
       <c r="D2" s="7"/>
       <c r="E2" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F2" s="5"/>
     </row>
@@ -3253,7 +3101,7 @@
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F3" s="5"/>
     </row>
@@ -3266,10 +3114,10 @@
         <v>37</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>116</v>
+        <v>86</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F4" s="5"/>
     </row>
@@ -3282,10 +3130,10 @@
         <v>37</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>116</v>
+        <v>86</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F5" s="5"/>
     </row>
@@ -3301,7 +3149,7 @@
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F6" s="5"/>
     </row>
@@ -3315,7 +3163,7 @@
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F7" s="5"/>
     </row>
@@ -3328,10 +3176,10 @@
         <v>39</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F8" s="5"/>
     </row>
@@ -3344,10 +3192,10 @@
         <v>39</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F9" s="5"/>
     </row>
@@ -3359,11 +3207,11 @@
         <v>0</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F10" s="5"/>
     </row>
@@ -3373,11 +3221,11 @@
         <v>0</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F11" s="5"/>
     </row>
@@ -3387,13 +3235,13 @@
         <v>1</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F12" s="5"/>
     </row>
@@ -3403,13 +3251,13 @@
         <v>1</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F13" s="5"/>
     </row>
@@ -3421,11 +3269,11 @@
         <v>0</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D14" s="7"/>
       <c r="E14" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F14" s="5"/>
     </row>
@@ -3435,11 +3283,11 @@
         <v>0</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D15" s="7"/>
       <c r="E15" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F15" s="5"/>
     </row>
@@ -3449,13 +3297,13 @@
         <v>1</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F16" s="5"/>
     </row>
@@ -3465,13 +3313,13 @@
         <v>1</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F17" s="5"/>
     </row>
@@ -3483,11 +3331,11 @@
         <v>0</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F18" s="5"/>
     </row>
@@ -3497,11 +3345,11 @@
         <v>0</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D19" s="7"/>
       <c r="E19" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F19" s="5"/>
     </row>
@@ -3511,13 +3359,13 @@
         <v>1</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F20" s="5"/>
     </row>
@@ -3527,13 +3375,13 @@
         <v>1</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F21" s="5"/>
     </row>
@@ -3545,11 +3393,11 @@
         <v>0</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F22" s="5"/>
     </row>
@@ -3559,11 +3407,11 @@
         <v>0</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D23" s="7"/>
       <c r="E23" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F23" s="5"/>
     </row>
@@ -3573,13 +3421,13 @@
         <v>1</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F24" s="5"/>
     </row>
@@ -3589,13 +3437,13 @@
         <v>1</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F25" s="5"/>
     </row>
@@ -3607,11 +3455,11 @@
         <v>0</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D26" s="7"/>
       <c r="E26" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F26" s="5"/>
     </row>
@@ -3621,11 +3469,11 @@
         <v>0</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D27" s="7"/>
       <c r="E27" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F27" s="5"/>
     </row>
@@ -3635,13 +3483,13 @@
         <v>1</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F28" s="5"/>
     </row>
@@ -3651,13 +3499,13 @@
         <v>1</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F29" s="5"/>
     </row>
@@ -3669,11 +3517,11 @@
         <v>0</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D30" s="7"/>
       <c r="E30" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F30" s="5"/>
     </row>
@@ -3683,11 +3531,11 @@
         <v>0</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D31" s="7"/>
       <c r="E31" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F31" s="5"/>
     </row>
@@ -3697,13 +3545,13 @@
         <v>1</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F32" s="5"/>
     </row>
@@ -3713,13 +3561,13 @@
         <v>1</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F33" s="5"/>
     </row>
@@ -3731,11 +3579,11 @@
         <v>0</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D34" s="7"/>
       <c r="E34" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F34" s="5"/>
     </row>
@@ -3745,11 +3593,11 @@
         <v>0</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F35" s="5"/>
     </row>
@@ -3759,13 +3607,13 @@
         <v>1</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>126</v>
+        <v>96</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F36" s="5"/>
     </row>
@@ -3775,13 +3623,13 @@
         <v>1</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>126</v>
+        <v>96</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F37" s="5"/>
     </row>
@@ -3793,11 +3641,11 @@
         <v>0</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="D38" s="7"/>
       <c r="E38" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F38" s="5"/>
     </row>
@@ -3807,11 +3655,11 @@
         <v>0</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="D39" s="7"/>
       <c r="E39" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F39" s="5"/>
     </row>
@@ -3821,13 +3669,13 @@
         <v>1</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>127</v>
+        <v>97</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F40" s="5"/>
     </row>
@@ -3837,13 +3685,13 @@
         <v>1</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>127</v>
+        <v>97</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F41" s="5"/>
     </row>
@@ -3855,11 +3703,11 @@
         <v>0</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D42" s="7"/>
       <c r="E42" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F42" s="5"/>
     </row>
@@ -3869,11 +3717,11 @@
         <v>0</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D43" s="7"/>
       <c r="E43" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F43" s="5"/>
     </row>
@@ -3883,13 +3731,13 @@
         <v>1</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>128</v>
+        <v>98</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F44" s="5"/>
     </row>
@@ -3899,13 +3747,13 @@
         <v>1</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>128</v>
+        <v>98</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F45" s="5"/>
     </row>
@@ -3917,11 +3765,11 @@
         <v>0</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D46" s="7"/>
       <c r="E46" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F46" s="5"/>
     </row>
@@ -3931,11 +3779,11 @@
         <v>0</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D47" s="7"/>
       <c r="E47" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F47" s="5"/>
     </row>
@@ -3945,13 +3793,13 @@
         <v>1</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>129</v>
+        <v>99</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F48" s="5"/>
     </row>
@@ -3961,13 +3809,13 @@
         <v>1</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>129</v>
+        <v>99</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F49" s="5"/>
     </row>
@@ -3979,11 +3827,11 @@
         <v>0</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="D50" s="7"/>
       <c r="E50" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F50" s="5"/>
     </row>
@@ -3993,11 +3841,11 @@
         <v>0</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="D51" s="7"/>
       <c r="E51" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F51" s="5"/>
     </row>
@@ -4007,13 +3855,13 @@
         <v>1</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F52" s="5"/>
     </row>
@@ -4023,13 +3871,13 @@
         <v>1</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F53" s="5"/>
     </row>
@@ -4041,11 +3889,11 @@
         <v>0</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="D54" s="7"/>
       <c r="E54" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F54" s="5"/>
     </row>
@@ -4055,11 +3903,11 @@
         <v>0</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="D55" s="7"/>
       <c r="E55" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F55" s="5"/>
     </row>
@@ -4069,13 +3917,13 @@
         <v>1</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>131</v>
+        <v>101</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F56" s="5"/>
     </row>
@@ -4085,13 +3933,13 @@
         <v>1</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>131</v>
+        <v>101</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F57" s="5"/>
     </row>
@@ -4103,11 +3951,11 @@
         <v>0</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="D58" s="7"/>
       <c r="E58" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F58" s="5"/>
     </row>
@@ -4117,11 +3965,11 @@
         <v>0</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="D59" s="7"/>
       <c r="E59" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F59" s="5"/>
     </row>
@@ -4131,13 +3979,13 @@
         <v>1</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>132</v>
+        <v>102</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F60" s="5"/>
     </row>
@@ -4147,13 +3995,13 @@
         <v>1</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>132</v>
+        <v>102</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F61" s="5"/>
     </row>
@@ -4165,11 +4013,11 @@
         <v>0</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="D62" s="7"/>
       <c r="E62" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F62" s="5"/>
     </row>
@@ -4179,11 +4027,11 @@
         <v>0</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="D63" s="7"/>
       <c r="E63" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F63" s="5"/>
     </row>
@@ -4193,13 +4041,13 @@
         <v>1</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>133</v>
+        <v>103</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F64" s="5"/>
     </row>
@@ -4209,13 +4057,13 @@
         <v>1</v>
       </c>
       <c r="C65" s="9" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>133</v>
+        <v>103</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F65" s="5"/>
     </row>
@@ -4227,11 +4075,11 @@
         <v>0</v>
       </c>
       <c r="C66" s="9" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="D66" s="7"/>
       <c r="E66" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F66" s="5"/>
     </row>
@@ -4241,11 +4089,11 @@
         <v>0</v>
       </c>
       <c r="C67" s="9" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="D67" s="7"/>
       <c r="E67" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F67" s="5"/>
     </row>
@@ -4255,13 +4103,13 @@
         <v>1</v>
       </c>
       <c r="C68" s="9" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>134</v>
+        <v>104</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F68" s="5"/>
     </row>
@@ -4271,13 +4119,13 @@
         <v>1</v>
       </c>
       <c r="C69" s="9" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>134</v>
+        <v>104</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F69" s="5"/>
     </row>
@@ -4289,11 +4137,11 @@
         <v>0</v>
       </c>
       <c r="C70" s="9" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="D70" s="7"/>
       <c r="E70" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F70" s="5"/>
     </row>
@@ -4303,11 +4151,11 @@
         <v>0</v>
       </c>
       <c r="C71" s="9" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="D71" s="7"/>
       <c r="E71" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F71" s="5"/>
     </row>
@@ -4317,13 +4165,13 @@
         <v>1</v>
       </c>
       <c r="C72" s="9" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>135</v>
+        <v>105</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F72" s="5"/>
     </row>
@@ -4333,13 +4181,13 @@
         <v>1</v>
       </c>
       <c r="C73" s="9" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>135</v>
+        <v>105</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F73" s="5"/>
     </row>
@@ -4351,11 +4199,11 @@
         <v>0</v>
       </c>
       <c r="C74" s="9" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="D74" s="7"/>
       <c r="E74" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F74" s="5"/>
     </row>
@@ -4365,11 +4213,11 @@
         <v>0</v>
       </c>
       <c r="C75" s="9" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="D75" s="7"/>
       <c r="E75" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F75" s="5"/>
     </row>
@@ -4379,13 +4227,13 @@
         <v>1</v>
       </c>
       <c r="C76" s="9" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>136</v>
+        <v>106</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F76" s="5"/>
     </row>
@@ -4395,13 +4243,13 @@
         <v>1</v>
       </c>
       <c r="C77" s="9" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>136</v>
+        <v>106</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F77" s="5"/>
     </row>
@@ -4413,11 +4261,11 @@
         <v>0</v>
       </c>
       <c r="C78" s="9" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="D78" s="7"/>
       <c r="E78" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F78" s="5"/>
     </row>
@@ -4427,11 +4275,11 @@
         <v>0</v>
       </c>
       <c r="C79" s="9" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="D79" s="7"/>
       <c r="E79" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F79" s="5"/>
     </row>
@@ -4441,13 +4289,13 @@
         <v>1</v>
       </c>
       <c r="C80" s="9" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>137</v>
+        <v>107</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F80" s="5"/>
     </row>
@@ -4457,13 +4305,13 @@
         <v>1</v>
       </c>
       <c r="C81" s="9" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>137</v>
+        <v>107</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F81" s="5"/>
     </row>
@@ -4475,11 +4323,11 @@
         <v>0</v>
       </c>
       <c r="C82" s="9" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="D82" s="7"/>
       <c r="E82" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F82" s="5"/>
     </row>
@@ -4489,11 +4337,11 @@
         <v>0</v>
       </c>
       <c r="C83" s="9" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="D83" s="7"/>
       <c r="E83" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F83" s="5"/>
     </row>
@@ -4503,13 +4351,13 @@
         <v>1</v>
       </c>
       <c r="C84" s="9" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>138</v>
+        <v>108</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F84" s="5"/>
     </row>
@@ -4519,13 +4367,13 @@
         <v>1</v>
       </c>
       <c r="C85" s="9" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>138</v>
+        <v>108</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F85" s="5"/>
     </row>
@@ -4537,11 +4385,11 @@
         <v>0</v>
       </c>
       <c r="C86" s="9" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="D86" s="7"/>
       <c r="E86" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F86" s="5"/>
     </row>
@@ -4551,11 +4399,11 @@
         <v>0</v>
       </c>
       <c r="C87" s="9" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="D87" s="7"/>
       <c r="E87" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F87" s="5"/>
     </row>
@@ -4565,13 +4413,13 @@
         <v>1</v>
       </c>
       <c r="C88" s="9" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F88" s="5"/>
     </row>
@@ -4581,13 +4429,13 @@
         <v>1</v>
       </c>
       <c r="C89" s="9" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="D89" s="10" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F89" s="5"/>
     </row>
@@ -4599,11 +4447,11 @@
         <v>0</v>
       </c>
       <c r="C90" s="9" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="D90" s="7"/>
       <c r="E90" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F90" s="5"/>
     </row>
@@ -4613,11 +4461,11 @@
         <v>0</v>
       </c>
       <c r="C91" s="9" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="D91" s="7"/>
       <c r="E91" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F91" s="5"/>
     </row>
@@ -4627,13 +4475,13 @@
         <v>1</v>
       </c>
       <c r="C92" s="9" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="D92" s="10" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F92" s="5"/>
     </row>
@@ -4643,13 +4491,13 @@
         <v>1</v>
       </c>
       <c r="C93" s="9" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="D93" s="10" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F93" s="5"/>
     </row>
@@ -4661,11 +4509,11 @@
         <v>0</v>
       </c>
       <c r="C94" s="9" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="D94" s="7"/>
       <c r="E94" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F94" s="5"/>
     </row>
@@ -4675,11 +4523,11 @@
         <v>0</v>
       </c>
       <c r="C95" s="9" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="D95" s="7"/>
       <c r="E95" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F95" s="5"/>
     </row>
@@ -4689,13 +4537,13 @@
         <v>1</v>
       </c>
       <c r="C96" s="9" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="D96" s="10" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F96" s="5"/>
     </row>
@@ -4705,13 +4553,13 @@
         <v>1</v>
       </c>
       <c r="C97" s="9" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="D97" s="10" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F97" s="5"/>
     </row>
@@ -4723,11 +4571,11 @@
         <v>0</v>
       </c>
       <c r="C98" s="9" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="D98" s="7"/>
       <c r="E98" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F98" s="5"/>
     </row>
@@ -4737,11 +4585,11 @@
         <v>0</v>
       </c>
       <c r="C99" s="9" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="D99" s="7"/>
       <c r="E99" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F99" s="5"/>
     </row>
@@ -4751,13 +4599,13 @@
         <v>1</v>
       </c>
       <c r="C100" s="9" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="D100" s="10" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F100" s="5"/>
     </row>
@@ -4767,13 +4615,13 @@
         <v>1</v>
       </c>
       <c r="C101" s="9" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="D101" s="10" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
       <c r="E101" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F101" s="5"/>
     </row>
@@ -4785,11 +4633,11 @@
         <v>0</v>
       </c>
       <c r="C102" s="9" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="D102" s="7"/>
       <c r="E102" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F102" s="5"/>
     </row>
@@ -4799,11 +4647,11 @@
         <v>0</v>
       </c>
       <c r="C103" s="9" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="D103" s="7"/>
       <c r="E103" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F103" s="5"/>
     </row>
@@ -4813,13 +4661,13 @@
         <v>1</v>
       </c>
       <c r="C104" s="9" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="D104" s="10" t="s">
-        <v>143</v>
+        <v>113</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F104" s="5"/>
     </row>
@@ -4829,13 +4677,13 @@
         <v>1</v>
       </c>
       <c r="C105" s="9" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="D105" s="10" t="s">
-        <v>143</v>
+        <v>113</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F105" s="5"/>
     </row>
@@ -4847,11 +4695,11 @@
         <v>0</v>
       </c>
       <c r="C106" s="9" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="D106" s="7"/>
       <c r="E106" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F106" s="5"/>
     </row>
@@ -4861,11 +4709,11 @@
         <v>0</v>
       </c>
       <c r="C107" s="9" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="D107" s="7"/>
       <c r="E107" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F107" s="5"/>
     </row>
@@ -4875,13 +4723,13 @@
         <v>1</v>
       </c>
       <c r="C108" s="9" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="D108" s="10" t="s">
-        <v>144</v>
+        <v>114</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F108" s="5"/>
     </row>
@@ -4891,13 +4739,13 @@
         <v>1</v>
       </c>
       <c r="C109" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D109" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="E109" s="5" t="s">
         <v>88</v>
-      </c>
-      <c r="D109" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="E109" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="F109" s="5"/>
     </row>
@@ -4909,11 +4757,11 @@
         <v>0</v>
       </c>
       <c r="C110" s="9" t="s">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="D110" s="7"/>
       <c r="E110" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F110" s="5"/>
     </row>
@@ -4923,11 +4771,11 @@
         <v>0</v>
       </c>
       <c r="C111" s="9" t="s">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="D111" s="7"/>
       <c r="E111" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F111" s="5"/>
     </row>
@@ -4937,13 +4785,13 @@
         <v>1</v>
       </c>
       <c r="C112" s="9" t="s">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="D112" s="7" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F112" s="5"/>
     </row>
@@ -4953,13 +4801,13 @@
         <v>1</v>
       </c>
       <c r="C113" s="9" t="s">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="D113" s="7" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="E113" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F113" s="5"/>
     </row>
@@ -4971,11 +4819,11 @@
         <v>0</v>
       </c>
       <c r="C114" s="9" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="D114" s="7"/>
       <c r="E114" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F114" s="5"/>
     </row>
@@ -4985,11 +4833,11 @@
         <v>0</v>
       </c>
       <c r="C115" s="9" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="D115" s="7"/>
       <c r="E115" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F115" s="5"/>
     </row>
@@ -4999,13 +4847,13 @@
         <v>1</v>
       </c>
       <c r="C116" s="9" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="D116" s="7" t="s">
-        <v>146</v>
+        <v>116</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F116" s="5"/>
     </row>
@@ -5015,13 +4863,13 @@
         <v>1</v>
       </c>
       <c r="C117" s="9" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="D117" s="7" t="s">
-        <v>146</v>
+        <v>116</v>
       </c>
       <c r="E117" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F117" s="5"/>
     </row>
@@ -5033,11 +4881,11 @@
         <v>0</v>
       </c>
       <c r="C118" s="9" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="D118" s="7"/>
       <c r="E118" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F118" s="5"/>
     </row>
@@ -5047,11 +4895,11 @@
         <v>0</v>
       </c>
       <c r="C119" s="9" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="D119" s="7"/>
       <c r="E119" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F119" s="5"/>
     </row>
@@ -5061,13 +4909,13 @@
         <v>1</v>
       </c>
       <c r="C120" s="9" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="D120" s="7" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F120" s="5"/>
     </row>
@@ -5077,13 +4925,13 @@
         <v>1</v>
       </c>
       <c r="C121" s="9" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="D121" s="7" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="E121" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F121" s="5"/>
     </row>
@@ -5095,11 +4943,11 @@
         <v>0</v>
       </c>
       <c r="C122" s="9" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="D122" s="7"/>
       <c r="E122" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F122" s="5"/>
     </row>
@@ -5109,11 +4957,11 @@
         <v>0</v>
       </c>
       <c r="C123" s="9" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="D123" s="7"/>
       <c r="E123" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F123" s="5"/>
     </row>
@@ -5123,13 +4971,13 @@
         <v>1</v>
       </c>
       <c r="C124" s="9" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="D124" s="7" t="s">
-        <v>148</v>
+        <v>118</v>
       </c>
       <c r="E124" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F124" s="5"/>
     </row>
@@ -5139,13 +4987,13 @@
         <v>1</v>
       </c>
       <c r="C125" s="9" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="D125" s="7" t="s">
-        <v>148</v>
+        <v>118</v>
       </c>
       <c r="E125" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F125" s="5"/>
     </row>
@@ -5157,11 +5005,11 @@
         <v>0</v>
       </c>
       <c r="C126" s="9" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="D126" s="7"/>
       <c r="E126" s="5" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="F126" s="5"/>
     </row>
@@ -5171,11 +5019,11 @@
         <v>0</v>
       </c>
       <c r="C127" s="9" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="D127" s="7"/>
       <c r="E127" s="5" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="F127" s="5"/>
     </row>
@@ -5185,13 +5033,13 @@
         <v>1</v>
       </c>
       <c r="C128" s="9" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="D128" s="7" t="s">
-        <v>149</v>
+        <v>119</v>
       </c>
       <c r="E128" s="5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="F128" s="5"/>
     </row>
@@ -5201,13 +5049,13 @@
         <v>1</v>
       </c>
       <c r="C129" s="9" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="D129" s="7" t="s">
-        <v>149</v>
+        <v>119</v>
       </c>
       <c r="E129" s="5" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="F129" s="5"/>
     </row>

</xml_diff>

<commit_message>
flat enable to counts
</commit_message>
<xml_diff>
--- a/silver_layer_data_validation_databrick_catalog/queries/validation_queries.xlsx
+++ b/silver_layer_data_validation_databrick_catalog/queries/validation_queries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6080" activeTab="2"/>
+    <workbookView windowWidth="19200" windowHeight="6080" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="db" sheetId="3" r:id="rId1"/>
@@ -3080,7 +3080,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>37</v>
@@ -3094,7 +3094,7 @@
     <row r="3" spans="1:6">
       <c r="A3" s="4"/>
       <c r="B3" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
infor table name is wrong
</commit_message>
<xml_diff>
--- a/silver_layer_data_validation_databrick_catalog/queries/validation_queries.xlsx
+++ b/silver_layer_data_validation_databrick_catalog/queries/validation_queries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6800" activeTab="3"/>
+    <workbookView windowWidth="19200" windowHeight="6800" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="db" sheetId="1" r:id="rId1"/>
@@ -320,7 +320,7 @@
     <t>infor_dimension_mapping_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\infor\infor_dimension_mapping_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\infor\infor_special_project_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>odoo_calender_event_base</t>

</xml_diff>

<commit_message>
Add offline sheets validation SQL queries
</commit_message>
<xml_diff>
--- a/silver_layer_data_validation_databrick_catalog/queries/validation_queries.xlsx
+++ b/silver_layer_data_validation_databrick_catalog/queries/validation_queries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6800" activeTab="2"/>
+    <workbookView windowWidth="19200" windowHeight="6080" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="db" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="162">
   <si>
     <t>db_name</t>
   </si>
@@ -317,7 +317,7 @@
     <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\withdrawal_base.sql</t>
   </si>
   <si>
-    <t>infor_dimension_mapping_base</t>
+    <t>infor_special_project_compare_bronze_silver</t>
   </si>
   <si>
     <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\infor\infor_special_project_compare_bronze_silver.sql</t>
@@ -338,34 +338,67 @@
     <t>offline_sheets_dapm_master_sheet</t>
   </si>
   <si>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\offline-sheets\converted to databricks\offline_sheets_dapm_master_sheet_compare_bronze_silver.sql</t>
+  </si>
+  <si>
     <t>offline_sheets_grtandgre_individuals</t>
   </si>
   <si>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\offline-sheets\converted to databricks\offline_sheets_grtandgre_individuals_compare_bronze_silver.sql</t>
+  </si>
+  <si>
     <t>offline_sheets_grtandgre_project_details</t>
   </si>
   <si>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\offline-sheets\converted to databricks\offline_sheets_grtandgre_project_details_compare_bronze_silver.sql</t>
+  </si>
+  <si>
     <t>offline_sheets_job_seeker_and_walkins_applications_tracker_v2</t>
   </si>
   <si>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\offline-sheets\converted to databricks\offline_sheets_job_seeker_and_walkins_applications_tracker_v2_compare_bronze_silver.sql</t>
+  </si>
+  <si>
     <t>offline_sheets_job_seeker_and_walkins_job_centers_details</t>
   </si>
   <si>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\offline-sheets\converted to databricks\offline_sheets_job_seeker_and_walkins_job_centers_details_compare_bronze_silver.sql</t>
+  </si>
+  <si>
     <t>offline_sheets_job_seeker_and_walkins_vacancies</t>
   </si>
   <si>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\offline-sheets\converted to databricks\offline_sheets_job_seeker_and_walkins_vacancies_compare_bronze_silver.sql</t>
+  </si>
+  <si>
     <t>offline_sheets_jobplus_csr</t>
   </si>
   <si>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\offline-sheets\converted to databricks\offline_sheets_jobplus_csr_compare_bronze_silver.sql</t>
+  </si>
+  <si>
     <t>offline_sheets_moic_active_and_deleted_crs</t>
   </si>
   <si>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\offline-sheets\converted to databricks\offline_sheets_moic_active_and_deleted_crs_compare_bronze_silver.sql</t>
+  </si>
+  <si>
     <t>offline_sheets_moic_owners_details</t>
   </si>
   <si>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\offline-sheets\converted to databricks\offline_sheets_moic_owners_details_compare_bronze_silver.sql</t>
+  </si>
+  <si>
     <t>offline_sheets_placement_and_approved_jobs_plus_applications</t>
   </si>
   <si>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\offline-sheets\converted to databricks\offline_sheets_placement_and_approved_jobs_plus_applications_compare_bronze_silver.sql</t>
+  </si>
+  <si>
     <t>offline_sheets_sio_employees</t>
+  </si>
+  <si>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\offline-sheets\converted to databricks\offline_sheets_sio_employees_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>business_keys</t>
@@ -1188,7 +1221,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1221,16 +1254,28 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
@@ -1795,100 +1840,100 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:9">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="I1" s="22" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="13">
         <v>8443</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="G2" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="12" t="s">
+      <c r="H2" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="13">
         <v>8443</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="12" t="s">
+      <c r="H3" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="13" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="13">
         <v>8443</v>
       </c>
       <c r="D4" s="10" t="s">
@@ -1897,27 +1942,27 @@
       <c r="E4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="12" t="s">
+      <c r="H4" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="13" t="s">
         <v>16</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="13">
         <v>8443</v>
       </c>
       <c r="D5" s="10" t="s">
@@ -1926,16 +1971,16 @@
       <c r="E5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="H5" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="12" t="s">
+      <c r="H5" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" s="13" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1951,25 +1996,25 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="4"/>
   <cols>
-    <col min="3" max="3" width="12.6363636363636" style="16" customWidth="1"/>
-    <col min="4" max="4" width="46.4545454545455" style="16" customWidth="1"/>
-    <col min="5" max="5" width="44.8181818181818" style="16" customWidth="1"/>
+    <col min="3" max="3" width="12.6363636363636" style="20" customWidth="1"/>
+    <col min="4" max="4" width="46.4545454545455" style="20" customWidth="1"/>
+    <col min="5" max="5" width="44.8181818181818" style="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="21" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2019,13 +2064,13 @@
   <dimension ref="A1:E126"/>
   <sheetFormatPr defaultColWidth="20.6363636363636" defaultRowHeight="14.5" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="2" width="3.72727272727273" style="2" customWidth="1"/>
-    <col min="3" max="3" width="27.9090909090909" style="2" customWidth="1"/>
-    <col min="4" max="4" width="120.181818181818" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="20.6363636363636" style="2" customWidth="1"/>
+    <col min="1" max="2" width="3.72727272727273" style="12" customWidth="1"/>
+    <col min="3" max="3" width="61.9090909090909" style="12" customWidth="1"/>
+    <col min="4" max="4" width="120.181818181818" style="12" customWidth="1"/>
+    <col min="5" max="16384" width="20.6363636363636" style="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="12" customHeight="1" spans="1:5">
+    <row r="1" s="2" customFormat="1" ht="12" customHeight="1" spans="1:5">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -2042,7 +2087,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1" spans="1:5">
+    <row r="2" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -2052,12 +2097,12 @@
       <c r="C2" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="13" t="s">
         <v>38</v>
       </c>
       <c r="E2" s="5"/>
     </row>
-    <row r="3" ht="29" customHeight="1" spans="1:5">
+    <row r="3" s="2" customFormat="1" ht="29" customHeight="1" spans="1:5">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -2067,12 +2112,12 @@
       <c r="C3" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="13" t="s">
         <v>40</v>
       </c>
       <c r="E3" s="5"/>
     </row>
-    <row r="4" ht="33" customHeight="1" spans="1:5">
+    <row r="4" s="2" customFormat="1" ht="33" customHeight="1" spans="1:5">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -2082,12 +2127,12 @@
       <c r="C4" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="13" t="s">
         <v>42</v>
       </c>
       <c r="E4" s="5"/>
     </row>
-    <row r="5" ht="30" customHeight="1" spans="1:5">
+    <row r="5" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -2097,12 +2142,12 @@
       <c r="C5" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="13" t="s">
         <v>44</v>
       </c>
       <c r="E5" s="5"/>
     </row>
-    <row r="6" ht="33" customHeight="1" spans="1:5">
+    <row r="6" s="2" customFormat="1" ht="33" customHeight="1" spans="1:5">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -2112,12 +2157,12 @@
       <c r="C6" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="13" t="s">
         <v>46</v>
       </c>
       <c r="E6" s="5"/>
     </row>
-    <row r="7" ht="32" customHeight="1" spans="1:5">
+    <row r="7" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -2127,27 +2172,27 @@
       <c r="C7" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="13" t="s">
         <v>48</v>
       </c>
       <c r="E7" s="5"/>
     </row>
-    <row r="8" ht="32" customHeight="1" spans="1:5">
+    <row r="8" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
       <c r="A8" s="5">
         <v>7</v>
       </c>
       <c r="B8" s="5">
         <v>0</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="13" t="s">
         <v>50</v>
       </c>
       <c r="E8" s="5"/>
     </row>
-    <row r="9" ht="32" customHeight="1" spans="1:5">
+    <row r="9" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -2157,12 +2202,12 @@
       <c r="C9" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="13" t="s">
         <v>52</v>
       </c>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" ht="32" customHeight="1" spans="1:5">
+    <row r="10" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -2172,202 +2217,202 @@
       <c r="C10" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="13" t="s">
         <v>54</v>
       </c>
       <c r="E10" s="5"/>
     </row>
-    <row r="11" ht="32" customHeight="1" spans="1:5">
+    <row r="11" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
       <c r="A11" s="5">
         <v>10</v>
       </c>
       <c r="B11" s="5">
         <v>1</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="13" t="s">
         <v>56</v>
       </c>
       <c r="E11" s="5"/>
     </row>
-    <row r="12" ht="32" customHeight="1" spans="1:5">
+    <row r="12" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
       <c r="A12" s="5">
         <v>11</v>
       </c>
       <c r="B12" s="5">
         <v>1</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="13" t="s">
         <v>58</v>
       </c>
       <c r="E12" s="5"/>
     </row>
-    <row r="13" ht="32" customHeight="1" spans="1:5">
+    <row r="13" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
       <c r="A13" s="5">
         <v>12</v>
       </c>
       <c r="B13" s="5">
         <v>0</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="13" t="s">
         <v>60</v>
       </c>
       <c r="E13" s="5"/>
     </row>
-    <row r="14" ht="32" customHeight="1" spans="1:5">
+    <row r="14" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
       <c r="A14" s="5">
         <v>13</v>
       </c>
       <c r="B14" s="5">
         <v>0</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="13" t="s">
         <v>62</v>
       </c>
       <c r="E14" s="5"/>
     </row>
-    <row r="15" ht="32" customHeight="1" spans="1:5">
+    <row r="15" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
       <c r="A15" s="5">
         <v>14</v>
       </c>
       <c r="B15" s="5">
         <v>0</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="13" t="s">
         <v>64</v>
       </c>
       <c r="E15" s="5"/>
     </row>
-    <row r="16" ht="32" customHeight="1" spans="1:5">
+    <row r="16" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
       <c r="A16" s="5">
         <v>15</v>
       </c>
       <c r="B16" s="5">
         <v>0</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="13" t="s">
         <v>66</v>
       </c>
       <c r="E16" s="5"/>
     </row>
-    <row r="17" ht="30" customHeight="1" spans="1:5">
+    <row r="17" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
       <c r="A17" s="5">
         <v>16</v>
       </c>
       <c r="B17" s="5">
         <v>0</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="13" t="s">
         <v>68</v>
       </c>
       <c r="E17" s="5"/>
     </row>
-    <row r="18" ht="30" customHeight="1" spans="1:5">
+    <row r="18" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
       <c r="A18" s="5">
         <v>17</v>
       </c>
       <c r="B18" s="5">
         <v>1</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="13" t="s">
         <v>70</v>
       </c>
       <c r="E18" s="5"/>
     </row>
-    <row r="19" ht="30" customHeight="1" spans="1:5">
+    <row r="19" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
       <c r="A19" s="5">
         <v>18</v>
       </c>
       <c r="B19" s="5">
         <v>0</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="13" t="s">
         <v>72</v>
       </c>
       <c r="E19" s="5"/>
     </row>
-    <row r="20" ht="30" customHeight="1" spans="1:5">
+    <row r="20" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
       <c r="A20" s="5">
         <v>19</v>
       </c>
       <c r="B20" s="5">
         <v>1</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="13" t="s">
         <v>74</v>
       </c>
       <c r="E20" s="5"/>
     </row>
-    <row r="21" ht="30" customHeight="1" spans="1:5">
+    <row r="21" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
       <c r="A21" s="5">
         <v>20</v>
       </c>
       <c r="B21" s="5">
         <v>1</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="13" t="s">
         <v>76</v>
       </c>
       <c r="E21" s="5"/>
     </row>
-    <row r="22" ht="30" customHeight="1" spans="1:5">
+    <row r="22" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
       <c r="A22" s="5">
         <v>21</v>
       </c>
       <c r="B22" s="5">
         <v>0</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D22" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="E22" s="12"/>
-    </row>
-    <row r="23" ht="30" customHeight="1" spans="1:5">
+      <c r="E22" s="13"/>
+    </row>
+    <row r="23" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
       <c r="A23" s="5">
         <v>22</v>
       </c>
       <c r="B23" s="5">
         <v>0</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="D23" s="13" t="s">
         <v>80</v>
       </c>
       <c r="E23" s="5"/>
@@ -2379,10 +2424,10 @@
       <c r="B24" s="5">
         <v>0</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="D24" s="12" t="s">
+      <c r="D24" s="13" t="s">
         <v>82</v>
       </c>
       <c r="E24" s="5"/>
@@ -2394,15 +2439,15 @@
       <c r="B25" s="5">
         <v>1</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="D25" s="12" t="s">
+      <c r="D25" s="13" t="s">
         <v>84</v>
       </c>
       <c r="E25" s="5"/>
     </row>
-    <row r="26" ht="27" customHeight="1" spans="1:5">
+    <row r="26" s="2" customFormat="1" ht="27" customHeight="1" spans="1:5">
       <c r="A26" s="5">
         <v>25</v>
       </c>
@@ -2412,12 +2457,12 @@
       <c r="C26" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D26" s="12" t="s">
+      <c r="D26" s="13" t="s">
         <v>86</v>
       </c>
       <c r="E26" s="5"/>
     </row>
-    <row r="27" ht="35" customHeight="1" spans="1:5">
+    <row r="27" s="2" customFormat="1" ht="35" customHeight="1" spans="1:5">
       <c r="A27" s="5">
         <v>26</v>
       </c>
@@ -2427,12 +2472,12 @@
       <c r="C27" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D27" s="12" t="s">
+      <c r="D27" s="13" t="s">
         <v>88</v>
       </c>
       <c r="E27" s="5"/>
     </row>
-    <row r="28" ht="35" customHeight="1" spans="1:5">
+    <row r="28" s="2" customFormat="1" ht="35" customHeight="1" spans="1:5">
       <c r="A28" s="5">
         <v>27</v>
       </c>
@@ -2442,27 +2487,27 @@
       <c r="C28" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="D28" s="12" t="s">
+      <c r="D28" s="13" t="s">
         <v>90</v>
       </c>
       <c r="E28" s="5"/>
     </row>
-    <row r="29" ht="35" customHeight="1" spans="1:5">
+    <row r="29" s="2" customFormat="1" ht="35" customHeight="1" spans="1:5">
       <c r="A29" s="5">
         <v>28</v>
       </c>
       <c r="B29" s="5">
         <v>0</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="D29" s="12" t="s">
+      <c r="D29" s="13" t="s">
         <v>92</v>
       </c>
       <c r="E29" s="5"/>
     </row>
-    <row r="30" ht="29" customHeight="1" spans="1:5">
+    <row r="30" s="2" customFormat="1" ht="29" customHeight="1" spans="1:5">
       <c r="A30" s="5">
         <v>29</v>
       </c>
@@ -2472,7 +2517,7 @@
       <c r="C30" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="D30" s="12" t="s">
+      <c r="D30" s="13" t="s">
         <v>94</v>
       </c>
       <c r="E30" s="5"/>
@@ -2484,10 +2529,10 @@
       <c r="B31" s="5">
         <v>1</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="D31" s="12" t="s">
+      <c r="D31" s="13" t="s">
         <v>96</v>
       </c>
       <c r="E31" s="5"/>
@@ -2502,7 +2547,7 @@
       <c r="C32" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="D32" s="12" t="s">
+      <c r="D32" s="13" t="s">
         <v>98</v>
       </c>
       <c r="E32" s="5"/>
@@ -2517,685 +2562,745 @@
       <c r="C33" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="D33" s="12" t="s">
+      <c r="D33" s="13" t="s">
         <v>100</v>
       </c>
       <c r="E33" s="5"/>
     </row>
     <row r="34" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
-      <c r="A34" s="5"/>
+      <c r="A34" s="5">
+        <v>33</v>
+      </c>
       <c r="B34" s="5">
         <v>0</v>
       </c>
       <c r="C34" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="D34" s="12"/>
+      <c r="D34" s="13" t="s">
+        <v>102</v>
+      </c>
       <c r="E34" s="5"/>
     </row>
     <row r="35" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
-      <c r="A35" s="5"/>
+      <c r="A35" s="5">
+        <v>34</v>
+      </c>
       <c r="B35" s="5">
         <v>0</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="D35" s="12"/>
+        <v>103</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>104</v>
+      </c>
       <c r="E35" s="5"/>
     </row>
     <row r="36" s="2" customFormat="1" ht="31" customHeight="1" spans="1:5">
-      <c r="A36" s="5"/>
+      <c r="A36" s="5">
+        <v>35</v>
+      </c>
       <c r="B36" s="5">
         <v>0</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="D36" s="12"/>
+        <v>105</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>106</v>
+      </c>
       <c r="E36" s="5"/>
     </row>
     <row r="37" s="2" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5"/>
+      <c r="A37" s="5">
+        <v>36</v>
+      </c>
+      <c r="B37" s="5">
+        <v>0</v>
+      </c>
       <c r="C37" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="D37" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>108</v>
+      </c>
       <c r="E37" s="5"/>
     </row>
     <row r="38" s="2" customFormat="1" ht="35" customHeight="1" spans="1:5">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
+      <c r="A38" s="5">
+        <v>37</v>
+      </c>
+      <c r="B38" s="5">
+        <v>0</v>
+      </c>
       <c r="C38" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="D38" s="12"/>
+        <v>109</v>
+      </c>
+      <c r="D38" s="13" t="s">
+        <v>110</v>
+      </c>
       <c r="E38" s="5"/>
     </row>
     <row r="39" s="2" customFormat="1" ht="29" customHeight="1" spans="1:5">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
+      <c r="A39" s="5">
+        <v>38</v>
+      </c>
+      <c r="B39" s="5">
+        <v>0</v>
+      </c>
       <c r="C39" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="D39" s="12"/>
+        <v>111</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>112</v>
+      </c>
       <c r="E39" s="5"/>
     </row>
     <row r="40" s="2" customFormat="1" ht="29" customHeight="1" spans="1:5">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
+      <c r="A40" s="5">
+        <v>39</v>
+      </c>
+      <c r="B40" s="5">
+        <v>0</v>
+      </c>
       <c r="C40" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="D40" s="12"/>
+        <v>113</v>
+      </c>
+      <c r="D40" s="13" t="s">
+        <v>114</v>
+      </c>
       <c r="E40" s="5"/>
     </row>
     <row r="41" s="2" customFormat="1" ht="36" customHeight="1" spans="1:5">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
+      <c r="A41" s="5">
+        <v>40</v>
+      </c>
+      <c r="B41" s="5">
+        <v>0</v>
+      </c>
       <c r="C41" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="D41" s="12"/>
+        <v>115</v>
+      </c>
+      <c r="D41" s="13" t="s">
+        <v>116</v>
+      </c>
       <c r="E41" s="5"/>
     </row>
     <row r="42" s="2" customFormat="1" ht="29" customHeight="1" spans="1:5">
-      <c r="A42" s="5"/>
-      <c r="B42" s="5"/>
+      <c r="A42" s="5">
+        <v>41</v>
+      </c>
+      <c r="B42" s="5">
+        <v>0</v>
+      </c>
       <c r="C42" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="D42" s="12"/>
+        <v>117</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>118</v>
+      </c>
       <c r="E42" s="5"/>
     </row>
     <row r="43" s="2" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A43" s="5"/>
-      <c r="B43" s="5"/>
+      <c r="A43" s="5">
+        <v>42</v>
+      </c>
+      <c r="B43" s="5">
+        <v>0</v>
+      </c>
       <c r="C43" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="D43" s="12"/>
+        <v>119</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>120</v>
+      </c>
       <c r="E43" s="5"/>
     </row>
     <row r="44" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5"/>
+      <c r="A44" s="5">
+        <v>43</v>
+      </c>
+      <c r="B44" s="5">
+        <v>0</v>
+      </c>
       <c r="C44" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="D44" s="12"/>
+        <v>121</v>
+      </c>
+      <c r="D44" s="13" t="s">
+        <v>122</v>
+      </c>
       <c r="E44" s="5"/>
     </row>
-    <row r="45" s="2" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="5"/>
-    </row>
-    <row r="46" s="2" customFormat="1" ht="29" customHeight="1" spans="1:5">
-      <c r="A46" s="5"/>
-      <c r="B46" s="5"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="5"/>
-    </row>
-    <row r="47" s="2" customFormat="1" ht="34" customHeight="1" spans="1:5">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="5"/>
-    </row>
-    <row r="48" s="2" customFormat="1" ht="31" customHeight="1" spans="1:5">
-      <c r="A48" s="5"/>
-      <c r="B48" s="5"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="5"/>
-    </row>
-    <row r="49" s="2" customFormat="1" ht="36" customHeight="1" spans="1:5">
-      <c r="A49" s="5"/>
-      <c r="B49" s="5"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="12"/>
-      <c r="E49" s="5"/>
-    </row>
-    <row r="50" s="2" customFormat="1" ht="31" customHeight="1" spans="1:5">
-      <c r="A50" s="5"/>
-      <c r="B50" s="5"/>
-      <c r="C50" s="13"/>
-      <c r="D50" s="12"/>
-      <c r="E50" s="5"/>
-    </row>
-    <row r="51" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A51" s="5"/>
-      <c r="B51" s="5"/>
-      <c r="C51" s="13"/>
-      <c r="D51" s="12"/>
-      <c r="E51" s="5"/>
-    </row>
-    <row r="52" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A52" s="5"/>
-      <c r="B52" s="5"/>
-      <c r="C52" s="13"/>
-      <c r="D52" s="12"/>
-      <c r="E52" s="5"/>
-    </row>
-    <row r="53" s="2" customFormat="1" ht="27" customHeight="1" spans="1:5">
-      <c r="A53" s="5"/>
-      <c r="B53" s="5"/>
-      <c r="C53" s="13"/>
-      <c r="D53" s="12"/>
-      <c r="E53" s="5"/>
-    </row>
-    <row r="54" s="2" customFormat="1" ht="31" customHeight="1" spans="1:5">
-      <c r="A54" s="5"/>
-      <c r="B54" s="5"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="12"/>
-      <c r="E54" s="5"/>
-    </row>
-    <row r="55" s="2" customFormat="1" ht="36" customHeight="1" spans="1:5">
-      <c r="A55" s="5"/>
-      <c r="B55" s="5"/>
-      <c r="C55" s="13"/>
-      <c r="D55" s="12"/>
-      <c r="E55" s="5"/>
-    </row>
-    <row r="56" s="2" customFormat="1" spans="1:5">
-      <c r="A56" s="5"/>
-      <c r="B56" s="5"/>
-      <c r="C56" s="13"/>
-      <c r="D56" s="12"/>
-      <c r="E56" s="5"/>
-    </row>
-    <row r="57" s="2" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A57" s="5"/>
-      <c r="B57" s="5"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="12"/>
-      <c r="E57" s="5"/>
-    </row>
-    <row r="58" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A58" s="5"/>
-      <c r="B58" s="5"/>
-      <c r="C58" s="13"/>
-      <c r="D58" s="12"/>
-      <c r="E58" s="5"/>
-    </row>
-    <row r="59" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A59" s="5"/>
-      <c r="B59" s="5"/>
-      <c r="C59" s="13"/>
-      <c r="D59" s="12"/>
-      <c r="E59" s="5"/>
-    </row>
-    <row r="60" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A60" s="5"/>
-      <c r="B60" s="5"/>
-      <c r="C60" s="13"/>
-      <c r="D60" s="12"/>
-      <c r="E60" s="5"/>
-    </row>
-    <row r="61" s="2" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A61" s="5"/>
-      <c r="B61" s="5"/>
-      <c r="C61" s="13"/>
-      <c r="D61" s="12"/>
-      <c r="E61" s="5"/>
-    </row>
-    <row r="62" s="2" customFormat="1" ht="29" customHeight="1" spans="1:5">
-      <c r="A62" s="5"/>
-      <c r="B62" s="5"/>
-      <c r="C62" s="13"/>
-      <c r="D62" s="12"/>
-      <c r="E62" s="5"/>
-    </row>
-    <row r="63" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
-      <c r="A63" s="5"/>
-      <c r="B63" s="5"/>
-      <c r="C63" s="13"/>
-      <c r="D63" s="12"/>
-      <c r="E63" s="5"/>
-    </row>
-    <row r="64" s="2" customFormat="1" ht="29" customHeight="1" spans="1:5">
-      <c r="A64" s="5"/>
-      <c r="B64" s="5"/>
-      <c r="C64" s="13"/>
-      <c r="D64" s="12"/>
-      <c r="E64" s="5"/>
-    </row>
-    <row r="65" s="2" customFormat="1" ht="31" customHeight="1" spans="1:5">
-      <c r="A65" s="5"/>
-      <c r="B65" s="5"/>
-      <c r="C65" s="13"/>
-      <c r="D65" s="12"/>
-      <c r="E65" s="5"/>
-    </row>
-    <row r="66" s="2" customFormat="1" ht="30" customHeight="1" spans="1:5">
-      <c r="A66" s="5"/>
-      <c r="B66" s="5"/>
-      <c r="C66" s="13"/>
-      <c r="D66" s="12"/>
-      <c r="E66" s="5"/>
-    </row>
-    <row r="67" s="2" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A67" s="5"/>
-      <c r="B67" s="5"/>
-      <c r="C67" s="13"/>
-      <c r="D67" s="12"/>
-      <c r="E67" s="5"/>
-    </row>
-    <row r="68" s="2" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A68" s="5"/>
-      <c r="B68" s="5"/>
-      <c r="C68" s="13"/>
-      <c r="D68" s="12"/>
-      <c r="E68" s="5"/>
-    </row>
-    <row r="69" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A69" s="5"/>
-      <c r="B69" s="5"/>
-      <c r="C69" s="13"/>
-      <c r="D69" s="12"/>
-      <c r="E69" s="5"/>
-    </row>
-    <row r="70" s="2" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A70" s="5"/>
-      <c r="B70" s="5"/>
-      <c r="C70" s="13"/>
-      <c r="D70" s="12"/>
-      <c r="E70" s="5"/>
-    </row>
-    <row r="71" s="2" customFormat="1" ht="31" customHeight="1" spans="1:5">
-      <c r="A71" s="5"/>
-      <c r="B71" s="5"/>
-      <c r="C71" s="13"/>
-      <c r="D71" s="12"/>
-      <c r="E71" s="5"/>
-    </row>
-    <row r="72" s="2" customFormat="1" spans="1:5">
-      <c r="A72" s="5"/>
-      <c r="B72" s="5"/>
-      <c r="C72" s="13"/>
-      <c r="D72" s="12"/>
-      <c r="E72" s="5"/>
-    </row>
-    <row r="73" s="2" customFormat="1" spans="1:5">
-      <c r="A73" s="5"/>
-      <c r="B73" s="5"/>
-      <c r="C73" s="13"/>
-      <c r="D73" s="12"/>
-      <c r="E73" s="5"/>
-    </row>
-    <row r="74" s="2" customFormat="1" spans="1:5">
-      <c r="A74" s="5"/>
-      <c r="B74" s="5"/>
-      <c r="C74" s="13"/>
-      <c r="D74" s="12"/>
-      <c r="E74" s="5"/>
-    </row>
-    <row r="75" s="2" customFormat="1" spans="1:5">
-      <c r="A75" s="5"/>
-      <c r="B75" s="5"/>
-      <c r="C75" s="13"/>
-      <c r="D75" s="12"/>
-      <c r="E75" s="5"/>
-    </row>
-    <row r="76" s="2" customFormat="1" spans="1:5">
-      <c r="A76" s="5"/>
-      <c r="B76" s="5"/>
-      <c r="C76" s="13"/>
-      <c r="D76" s="12"/>
-      <c r="E76" s="5"/>
-    </row>
-    <row r="77" s="2" customFormat="1" spans="1:5">
-      <c r="A77" s="5"/>
-      <c r="B77" s="5"/>
-      <c r="C77" s="13"/>
-      <c r="D77" s="12"/>
-      <c r="E77" s="5"/>
+    <row r="45" s="12" customFormat="1" ht="33" customHeight="1" spans="1:5">
+      <c r="A45" s="15"/>
+      <c r="B45" s="15"/>
+      <c r="D45" s="16"/>
+      <c r="E45" s="15"/>
+    </row>
+    <row r="46" s="12" customFormat="1" ht="29" customHeight="1" spans="1:5">
+      <c r="A46" s="15"/>
+      <c r="B46" s="15"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="15"/>
+    </row>
+    <row r="47" s="12" customFormat="1" ht="34" customHeight="1" spans="1:5">
+      <c r="A47" s="15"/>
+      <c r="B47" s="15"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="15"/>
+    </row>
+    <row r="48" s="12" customFormat="1" ht="31" customHeight="1" spans="1:5">
+      <c r="A48" s="15"/>
+      <c r="B48" s="15"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="15"/>
+    </row>
+    <row r="49" s="12" customFormat="1" ht="36" customHeight="1" spans="1:5">
+      <c r="A49" s="15"/>
+      <c r="B49" s="15"/>
+      <c r="C49" s="17"/>
+      <c r="D49" s="16"/>
+      <c r="E49" s="15"/>
+    </row>
+    <row r="50" s="12" customFormat="1" ht="31" customHeight="1" spans="1:5">
+      <c r="A50" s="15"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="16"/>
+      <c r="E50" s="15"/>
+    </row>
+    <row r="51" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
+      <c r="A51" s="15"/>
+      <c r="B51" s="15"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="16"/>
+      <c r="E51" s="15"/>
+    </row>
+    <row r="52" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
+      <c r="A52" s="15"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="18"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="15"/>
+    </row>
+    <row r="53" s="12" customFormat="1" ht="27" customHeight="1" spans="1:5">
+      <c r="A53" s="15"/>
+      <c r="B53" s="15"/>
+      <c r="C53" s="18"/>
+      <c r="D53" s="16"/>
+      <c r="E53" s="15"/>
+    </row>
+    <row r="54" s="12" customFormat="1" ht="31" customHeight="1" spans="1:5">
+      <c r="A54" s="15"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="16"/>
+      <c r="E54" s="15"/>
+    </row>
+    <row r="55" s="12" customFormat="1" ht="36" customHeight="1" spans="1:5">
+      <c r="A55" s="15"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="15"/>
+    </row>
+    <row r="56" s="12" customFormat="1" spans="1:5">
+      <c r="A56" s="15"/>
+      <c r="B56" s="15"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="16"/>
+      <c r="E56" s="15"/>
+    </row>
+    <row r="57" s="12" customFormat="1" ht="33" customHeight="1" spans="1:5">
+      <c r="A57" s="15"/>
+      <c r="B57" s="15"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="16"/>
+      <c r="E57" s="15"/>
+    </row>
+    <row r="58" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
+      <c r="A58" s="15"/>
+      <c r="B58" s="15"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="16"/>
+      <c r="E58" s="15"/>
+    </row>
+    <row r="59" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
+      <c r="A59" s="15"/>
+      <c r="B59" s="15"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="16"/>
+      <c r="E59" s="15"/>
+    </row>
+    <row r="60" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
+      <c r="A60" s="15"/>
+      <c r="B60" s="15"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="16"/>
+      <c r="E60" s="15"/>
+    </row>
+    <row r="61" s="12" customFormat="1" ht="33" customHeight="1" spans="1:5">
+      <c r="A61" s="15"/>
+      <c r="B61" s="15"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="16"/>
+      <c r="E61" s="15"/>
+    </row>
+    <row r="62" s="12" customFormat="1" ht="29" customHeight="1" spans="1:5">
+      <c r="A62" s="15"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="16"/>
+      <c r="E62" s="15"/>
+    </row>
+    <row r="63" s="12" customFormat="1" ht="30" customHeight="1" spans="1:5">
+      <c r="A63" s="15"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="18"/>
+      <c r="D63" s="16"/>
+      <c r="E63" s="15"/>
+    </row>
+    <row r="64" s="12" customFormat="1" ht="29" customHeight="1" spans="1:5">
+      <c r="A64" s="15"/>
+      <c r="B64" s="15"/>
+      <c r="C64" s="18"/>
+      <c r="D64" s="16"/>
+      <c r="E64" s="15"/>
+    </row>
+    <row r="65" s="12" customFormat="1" ht="31" customHeight="1" spans="1:5">
+      <c r="A65" s="15"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="18"/>
+      <c r="D65" s="16"/>
+      <c r="E65" s="15"/>
+    </row>
+    <row r="66" s="12" customFormat="1" ht="30" customHeight="1" spans="1:5">
+      <c r="A66" s="15"/>
+      <c r="B66" s="15"/>
+      <c r="C66" s="18"/>
+      <c r="D66" s="16"/>
+      <c r="E66" s="15"/>
+    </row>
+    <row r="67" s="12" customFormat="1" ht="33" customHeight="1" spans="1:5">
+      <c r="A67" s="15"/>
+      <c r="B67" s="15"/>
+      <c r="C67" s="18"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="15"/>
+    </row>
+    <row r="68" s="12" customFormat="1" ht="33" customHeight="1" spans="1:5">
+      <c r="A68" s="15"/>
+      <c r="B68" s="15"/>
+      <c r="C68" s="18"/>
+      <c r="D68" s="16"/>
+      <c r="E68" s="15"/>
+    </row>
+    <row r="69" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
+      <c r="A69" s="15"/>
+      <c r="B69" s="15"/>
+      <c r="C69" s="18"/>
+      <c r="D69" s="16"/>
+      <c r="E69" s="15"/>
+    </row>
+    <row r="70" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
+      <c r="A70" s="15"/>
+      <c r="B70" s="15"/>
+      <c r="C70" s="18"/>
+      <c r="D70" s="16"/>
+      <c r="E70" s="15"/>
+    </row>
+    <row r="71" s="12" customFormat="1" ht="31" customHeight="1" spans="1:5">
+      <c r="A71" s="15"/>
+      <c r="B71" s="15"/>
+      <c r="C71" s="18"/>
+      <c r="D71" s="16"/>
+      <c r="E71" s="15"/>
+    </row>
+    <row r="72" s="12" customFormat="1" spans="1:5">
+      <c r="A72" s="15"/>
+      <c r="B72" s="15"/>
+      <c r="C72" s="18"/>
+      <c r="D72" s="16"/>
+      <c r="E72" s="15"/>
+    </row>
+    <row r="73" s="12" customFormat="1" spans="1:5">
+      <c r="A73" s="15"/>
+      <c r="B73" s="15"/>
+      <c r="C73" s="18"/>
+      <c r="D73" s="16"/>
+      <c r="E73" s="15"/>
+    </row>
+    <row r="74" s="12" customFormat="1" spans="1:5">
+      <c r="A74" s="15"/>
+      <c r="B74" s="15"/>
+      <c r="C74" s="18"/>
+      <c r="D74" s="16"/>
+      <c r="E74" s="15"/>
+    </row>
+    <row r="75" s="12" customFormat="1" spans="1:5">
+      <c r="A75" s="15"/>
+      <c r="B75" s="15"/>
+      <c r="C75" s="18"/>
+      <c r="D75" s="16"/>
+      <c r="E75" s="15"/>
+    </row>
+    <row r="76" s="12" customFormat="1" spans="1:5">
+      <c r="A76" s="15"/>
+      <c r="B76" s="15"/>
+      <c r="C76" s="18"/>
+      <c r="D76" s="16"/>
+      <c r="E76" s="15"/>
+    </row>
+    <row r="77" s="12" customFormat="1" spans="1:5">
+      <c r="A77" s="15"/>
+      <c r="B77" s="15"/>
+      <c r="C77" s="18"/>
+      <c r="D77" s="16"/>
+      <c r="E77" s="15"/>
     </row>
     <row r="78" spans="1:5">
-      <c r="A78" s="5"/>
-      <c r="B78" s="5"/>
-      <c r="C78" s="13"/>
-      <c r="D78" s="12"/>
-      <c r="E78" s="5"/>
+      <c r="A78" s="15"/>
+      <c r="B78" s="15"/>
+      <c r="C78" s="18"/>
+      <c r="D78" s="16"/>
+      <c r="E78" s="15"/>
     </row>
     <row r="79" spans="1:5">
-      <c r="A79" s="5"/>
-      <c r="B79" s="5"/>
-      <c r="C79" s="13"/>
-      <c r="D79" s="12"/>
-      <c r="E79" s="5"/>
+      <c r="A79" s="15"/>
+      <c r="B79" s="15"/>
+      <c r="C79" s="18"/>
+      <c r="D79" s="16"/>
+      <c r="E79" s="15"/>
     </row>
     <row r="80" spans="1:5">
-      <c r="A80" s="5"/>
-      <c r="B80" s="5"/>
-      <c r="C80" s="13"/>
-      <c r="D80" s="12"/>
-      <c r="E80" s="5"/>
+      <c r="A80" s="15"/>
+      <c r="B80" s="15"/>
+      <c r="C80" s="18"/>
+      <c r="D80" s="16"/>
+      <c r="E80" s="15"/>
     </row>
     <row r="81" spans="1:5">
-      <c r="A81" s="5"/>
-      <c r="B81" s="5"/>
-      <c r="C81" s="13"/>
-      <c r="D81" s="12"/>
-      <c r="E81" s="5"/>
+      <c r="A81" s="15"/>
+      <c r="B81" s="15"/>
+      <c r="C81" s="18"/>
+      <c r="D81" s="16"/>
+      <c r="E81" s="15"/>
     </row>
     <row r="82" spans="1:5">
-      <c r="A82" s="5"/>
-      <c r="B82" s="5"/>
-      <c r="C82" s="13"/>
-      <c r="D82" s="12"/>
-      <c r="E82" s="5"/>
+      <c r="A82" s="15"/>
+      <c r="B82" s="15"/>
+      <c r="C82" s="18"/>
+      <c r="D82" s="16"/>
+      <c r="E82" s="15"/>
     </row>
     <row r="83" spans="1:5">
-      <c r="A83" s="5"/>
-      <c r="B83" s="5"/>
-      <c r="C83" s="13"/>
-      <c r="D83" s="12"/>
-      <c r="E83" s="5"/>
+      <c r="A83" s="15"/>
+      <c r="B83" s="15"/>
+      <c r="C83" s="18"/>
+      <c r="D83" s="16"/>
+      <c r="E83" s="15"/>
     </row>
     <row r="84" spans="1:5">
-      <c r="A84" s="5"/>
-      <c r="B84" s="5"/>
-      <c r="C84" s="13"/>
-      <c r="D84" s="12"/>
-      <c r="E84" s="5"/>
+      <c r="A84" s="15"/>
+      <c r="B84" s="15"/>
+      <c r="C84" s="18"/>
+      <c r="D84" s="16"/>
+      <c r="E84" s="15"/>
     </row>
     <row r="85" spans="1:5">
-      <c r="A85" s="5"/>
-      <c r="B85" s="5"/>
-      <c r="C85" s="13"/>
-      <c r="D85" s="12"/>
-      <c r="E85" s="5"/>
+      <c r="A85" s="15"/>
+      <c r="B85" s="15"/>
+      <c r="C85" s="18"/>
+      <c r="D85" s="16"/>
+      <c r="E85" s="15"/>
     </row>
     <row r="86" spans="1:5">
-      <c r="A86" s="5"/>
-      <c r="B86" s="5"/>
-      <c r="C86" s="13"/>
-      <c r="D86" s="12"/>
-      <c r="E86" s="5"/>
+      <c r="A86" s="15"/>
+      <c r="B86" s="15"/>
+      <c r="C86" s="18"/>
+      <c r="D86" s="16"/>
+      <c r="E86" s="15"/>
     </row>
     <row r="87" spans="1:5">
-      <c r="A87" s="5"/>
-      <c r="B87" s="5"/>
-      <c r="C87" s="13"/>
-      <c r="D87" s="12"/>
-      <c r="E87" s="5"/>
+      <c r="A87" s="15"/>
+      <c r="B87" s="15"/>
+      <c r="C87" s="18"/>
+      <c r="D87" s="16"/>
+      <c r="E87" s="15"/>
     </row>
     <row r="88" spans="1:5">
-      <c r="A88" s="5"/>
-      <c r="B88" s="5"/>
-      <c r="C88" s="13"/>
-      <c r="D88" s="12"/>
-      <c r="E88" s="5"/>
+      <c r="A88" s="15"/>
+      <c r="B88" s="15"/>
+      <c r="C88" s="18"/>
+      <c r="D88" s="16"/>
+      <c r="E88" s="15"/>
     </row>
     <row r="89" spans="1:5">
-      <c r="A89" s="5"/>
-      <c r="B89" s="5"/>
-      <c r="C89" s="13"/>
-      <c r="D89" s="12"/>
-      <c r="E89" s="5"/>
+      <c r="A89" s="15"/>
+      <c r="B89" s="15"/>
+      <c r="C89" s="18"/>
+      <c r="D89" s="16"/>
+      <c r="E89" s="15"/>
     </row>
     <row r="90" spans="1:5">
-      <c r="A90" s="5"/>
-      <c r="B90" s="5"/>
-      <c r="C90" s="13"/>
-      <c r="D90" s="12"/>
-      <c r="E90" s="5"/>
+      <c r="A90" s="15"/>
+      <c r="B90" s="15"/>
+      <c r="C90" s="18"/>
+      <c r="D90" s="16"/>
+      <c r="E90" s="15"/>
     </row>
     <row r="91" spans="1:5">
-      <c r="A91" s="5"/>
-      <c r="B91" s="5"/>
-      <c r="C91" s="13"/>
-      <c r="D91" s="12"/>
-      <c r="E91" s="5"/>
+      <c r="A91" s="15"/>
+      <c r="B91" s="15"/>
+      <c r="C91" s="18"/>
+      <c r="D91" s="16"/>
+      <c r="E91" s="15"/>
     </row>
     <row r="92" spans="1:5">
-      <c r="A92" s="5"/>
-      <c r="B92" s="5"/>
-      <c r="C92" s="13"/>
-      <c r="D92" s="12"/>
-      <c r="E92" s="5"/>
+      <c r="A92" s="15"/>
+      <c r="B92" s="15"/>
+      <c r="C92" s="18"/>
+      <c r="D92" s="16"/>
+      <c r="E92" s="15"/>
     </row>
     <row r="93" spans="1:5">
-      <c r="A93" s="5"/>
-      <c r="B93" s="5"/>
-      <c r="C93" s="13"/>
-      <c r="D93" s="12"/>
-      <c r="E93" s="5"/>
+      <c r="A93" s="15"/>
+      <c r="B93" s="15"/>
+      <c r="C93" s="18"/>
+      <c r="D93" s="16"/>
+      <c r="E93" s="15"/>
     </row>
     <row r="94" spans="1:5">
-      <c r="A94" s="5"/>
-      <c r="B94" s="5"/>
-      <c r="C94" s="13"/>
-      <c r="D94" s="12"/>
-      <c r="E94" s="5"/>
+      <c r="A94" s="15"/>
+      <c r="B94" s="15"/>
+      <c r="C94" s="18"/>
+      <c r="D94" s="16"/>
+      <c r="E94" s="15"/>
     </row>
     <row r="95" spans="1:5">
-      <c r="A95" s="5"/>
-      <c r="B95" s="5"/>
-      <c r="C95" s="13"/>
-      <c r="D95" s="12"/>
-      <c r="E95" s="5"/>
+      <c r="A95" s="15"/>
+      <c r="B95" s="15"/>
+      <c r="C95" s="18"/>
+      <c r="D95" s="16"/>
+      <c r="E95" s="15"/>
     </row>
     <row r="96" spans="1:5">
-      <c r="A96" s="5"/>
-      <c r="B96" s="5"/>
-      <c r="C96" s="13"/>
-      <c r="D96" s="12"/>
-      <c r="E96" s="5"/>
+      <c r="A96" s="15"/>
+      <c r="B96" s="15"/>
+      <c r="C96" s="18"/>
+      <c r="D96" s="16"/>
+      <c r="E96" s="15"/>
     </row>
     <row r="97" spans="1:5">
-      <c r="A97" s="5"/>
-      <c r="B97" s="5"/>
-      <c r="C97" s="13"/>
-      <c r="D97" s="12"/>
-      <c r="E97" s="5"/>
+      <c r="A97" s="15"/>
+      <c r="B97" s="15"/>
+      <c r="C97" s="18"/>
+      <c r="D97" s="16"/>
+      <c r="E97" s="15"/>
     </row>
     <row r="98" spans="1:5">
-      <c r="A98" s="5"/>
-      <c r="B98" s="5"/>
-      <c r="C98" s="13"/>
-      <c r="D98" s="12"/>
-      <c r="E98" s="5"/>
+      <c r="A98" s="15"/>
+      <c r="B98" s="15"/>
+      <c r="C98" s="18"/>
+      <c r="D98" s="16"/>
+      <c r="E98" s="15"/>
     </row>
     <row r="99" spans="1:5">
-      <c r="A99" s="5"/>
-      <c r="B99" s="5"/>
-      <c r="C99" s="13"/>
-      <c r="D99" s="12"/>
-      <c r="E99" s="5"/>
+      <c r="A99" s="15"/>
+      <c r="B99" s="15"/>
+      <c r="C99" s="18"/>
+      <c r="D99" s="16"/>
+      <c r="E99" s="15"/>
     </row>
     <row r="100" spans="1:5">
-      <c r="A100" s="5"/>
-      <c r="B100" s="5"/>
-      <c r="C100" s="13"/>
-      <c r="D100" s="12"/>
-      <c r="E100" s="5"/>
+      <c r="A100" s="15"/>
+      <c r="B100" s="15"/>
+      <c r="C100" s="18"/>
+      <c r="D100" s="16"/>
+      <c r="E100" s="15"/>
     </row>
     <row r="101" spans="1:5">
-      <c r="A101" s="5"/>
-      <c r="B101" s="5"/>
-      <c r="C101" s="13"/>
-      <c r="D101" s="12"/>
-      <c r="E101" s="5"/>
+      <c r="A101" s="15"/>
+      <c r="B101" s="15"/>
+      <c r="C101" s="18"/>
+      <c r="D101" s="16"/>
+      <c r="E101" s="15"/>
     </row>
     <row r="102" spans="1:5">
-      <c r="A102" s="5"/>
-      <c r="B102" s="5"/>
-      <c r="C102" s="13"/>
-      <c r="D102" s="12"/>
-      <c r="E102" s="5"/>
+      <c r="A102" s="15"/>
+      <c r="B102" s="15"/>
+      <c r="C102" s="18"/>
+      <c r="D102" s="16"/>
+      <c r="E102" s="15"/>
     </row>
     <row r="103" spans="1:5">
-      <c r="A103" s="5"/>
-      <c r="B103" s="5"/>
-      <c r="C103" s="13"/>
-      <c r="D103" s="12"/>
-      <c r="E103" s="5"/>
+      <c r="A103" s="15"/>
+      <c r="B103" s="15"/>
+      <c r="C103" s="18"/>
+      <c r="D103" s="16"/>
+      <c r="E103" s="15"/>
     </row>
     <row r="104" spans="1:5">
-      <c r="A104" s="5"/>
-      <c r="B104" s="5"/>
-      <c r="C104" s="13"/>
-      <c r="D104" s="12"/>
-      <c r="E104" s="5"/>
+      <c r="A104" s="15"/>
+      <c r="B104" s="15"/>
+      <c r="C104" s="18"/>
+      <c r="D104" s="16"/>
+      <c r="E104" s="15"/>
     </row>
     <row r="105" spans="1:5">
-      <c r="A105" s="5"/>
-      <c r="B105" s="5"/>
-      <c r="C105" s="13"/>
-      <c r="D105" s="12"/>
-      <c r="E105" s="5"/>
+      <c r="A105" s="15"/>
+      <c r="B105" s="15"/>
+      <c r="C105" s="18"/>
+      <c r="D105" s="16"/>
+      <c r="E105" s="15"/>
     </row>
     <row r="106" spans="1:5">
-      <c r="A106" s="5"/>
-      <c r="B106" s="5"/>
-      <c r="C106" s="13"/>
-      <c r="D106" s="12"/>
-      <c r="E106" s="5"/>
+      <c r="A106" s="15"/>
+      <c r="B106" s="15"/>
+      <c r="C106" s="18"/>
+      <c r="D106" s="16"/>
+      <c r="E106" s="15"/>
     </row>
     <row r="107" spans="1:5">
-      <c r="A107" s="5"/>
-      <c r="B107" s="5"/>
-      <c r="C107" s="13"/>
-      <c r="D107" s="12"/>
-      <c r="E107" s="5"/>
+      <c r="A107" s="15"/>
+      <c r="B107" s="15"/>
+      <c r="C107" s="18"/>
+      <c r="D107" s="16"/>
+      <c r="E107" s="15"/>
     </row>
     <row r="108" spans="1:5">
-      <c r="A108" s="5"/>
-      <c r="B108" s="5"/>
-      <c r="C108" s="13"/>
-      <c r="D108" s="12"/>
-      <c r="E108" s="5"/>
+      <c r="A108" s="15"/>
+      <c r="B108" s="15"/>
+      <c r="C108" s="18"/>
+      <c r="D108" s="16"/>
+      <c r="E108" s="15"/>
     </row>
     <row r="109" spans="1:5">
-      <c r="A109" s="5"/>
-      <c r="B109" s="5"/>
-      <c r="C109" s="13"/>
-      <c r="D109" s="12"/>
-      <c r="E109" s="5"/>
+      <c r="A109" s="15"/>
+      <c r="B109" s="15"/>
+      <c r="C109" s="18"/>
+      <c r="D109" s="16"/>
+      <c r="E109" s="15"/>
     </row>
     <row r="110" spans="1:5">
-      <c r="A110" s="5"/>
-      <c r="B110" s="5"/>
-      <c r="C110" s="13"/>
-      <c r="D110" s="12"/>
-      <c r="E110" s="5"/>
+      <c r="A110" s="15"/>
+      <c r="B110" s="15"/>
+      <c r="C110" s="18"/>
+      <c r="D110" s="16"/>
+      <c r="E110" s="15"/>
     </row>
     <row r="111" spans="1:5">
-      <c r="A111" s="5"/>
-      <c r="B111" s="5"/>
-      <c r="C111" s="13"/>
-      <c r="D111" s="12"/>
-      <c r="E111" s="5"/>
+      <c r="A111" s="15"/>
+      <c r="B111" s="15"/>
+      <c r="C111" s="18"/>
+      <c r="D111" s="16"/>
+      <c r="E111" s="15"/>
     </row>
     <row r="112" spans="1:5">
-      <c r="A112" s="5"/>
-      <c r="B112" s="5"/>
-      <c r="C112" s="13"/>
-      <c r="D112" s="12"/>
-      <c r="E112" s="5"/>
+      <c r="A112" s="15"/>
+      <c r="B112" s="15"/>
+      <c r="C112" s="18"/>
+      <c r="D112" s="16"/>
+      <c r="E112" s="15"/>
     </row>
     <row r="113" spans="1:5">
-      <c r="A113" s="5"/>
-      <c r="B113" s="5"/>
-      <c r="C113" s="13"/>
-      <c r="D113" s="12"/>
-      <c r="E113" s="5"/>
+      <c r="A113" s="15"/>
+      <c r="B113" s="15"/>
+      <c r="C113" s="18"/>
+      <c r="D113" s="16"/>
+      <c r="E113" s="15"/>
     </row>
     <row r="114" spans="1:5">
-      <c r="A114" s="5"/>
-      <c r="B114" s="5"/>
-      <c r="C114" s="13"/>
-      <c r="D114" s="12"/>
-      <c r="E114" s="5"/>
+      <c r="A114" s="15"/>
+      <c r="B114" s="15"/>
+      <c r="C114" s="18"/>
+      <c r="D114" s="16"/>
+      <c r="E114" s="15"/>
     </row>
     <row r="115" spans="1:5">
-      <c r="A115" s="5"/>
-      <c r="B115" s="5"/>
-      <c r="C115" s="13"/>
-      <c r="D115" s="12"/>
-      <c r="E115" s="5"/>
+      <c r="A115" s="15"/>
+      <c r="B115" s="15"/>
+      <c r="C115" s="18"/>
+      <c r="D115" s="16"/>
+      <c r="E115" s="15"/>
     </row>
     <row r="116" spans="1:5">
-      <c r="A116" s="5"/>
-      <c r="B116" s="5"/>
-      <c r="C116" s="13"/>
-      <c r="D116" s="12"/>
-      <c r="E116" s="5"/>
+      <c r="A116" s="15"/>
+      <c r="B116" s="15"/>
+      <c r="C116" s="18"/>
+      <c r="D116" s="16"/>
+      <c r="E116" s="15"/>
     </row>
     <row r="117" spans="1:5">
-      <c r="A117" s="5"/>
-      <c r="B117" s="5"/>
-      <c r="C117" s="13"/>
-      <c r="D117" s="12"/>
-      <c r="E117" s="5"/>
+      <c r="A117" s="15"/>
+      <c r="B117" s="15"/>
+      <c r="C117" s="18"/>
+      <c r="D117" s="16"/>
+      <c r="E117" s="15"/>
     </row>
     <row r="118" spans="1:5">
-      <c r="A118" s="5"/>
-      <c r="B118" s="5"/>
-      <c r="C118" s="13"/>
-      <c r="D118" s="12"/>
-      <c r="E118" s="5"/>
+      <c r="A118" s="15"/>
+      <c r="B118" s="15"/>
+      <c r="C118" s="18"/>
+      <c r="D118" s="16"/>
+      <c r="E118" s="15"/>
     </row>
     <row r="119" spans="1:5">
-      <c r="A119" s="5"/>
-      <c r="B119" s="5"/>
-      <c r="C119" s="13"/>
-      <c r="D119" s="12"/>
-      <c r="E119" s="5"/>
+      <c r="A119" s="15"/>
+      <c r="B119" s="15"/>
+      <c r="C119" s="18"/>
+      <c r="D119" s="16"/>
+      <c r="E119" s="15"/>
     </row>
     <row r="120" spans="1:5">
-      <c r="A120" s="5"/>
-      <c r="B120" s="5"/>
-      <c r="C120" s="13"/>
-      <c r="D120" s="12"/>
-      <c r="E120" s="5"/>
+      <c r="A120" s="15"/>
+      <c r="B120" s="15"/>
+      <c r="C120" s="18"/>
+      <c r="D120" s="16"/>
+      <c r="E120" s="15"/>
     </row>
     <row r="121" spans="1:5">
-      <c r="A121" s="5"/>
-      <c r="B121" s="5"/>
-      <c r="C121" s="13"/>
-      <c r="D121" s="12"/>
-      <c r="E121" s="5"/>
+      <c r="A121" s="15"/>
+      <c r="B121" s="15"/>
+      <c r="C121" s="18"/>
+      <c r="D121" s="16"/>
+      <c r="E121" s="15"/>
     </row>
     <row r="122" spans="1:5">
-      <c r="A122" s="5"/>
-      <c r="B122" s="5"/>
-      <c r="C122" s="13"/>
-      <c r="D122" s="12"/>
-      <c r="E122" s="5"/>
+      <c r="A122" s="15"/>
+      <c r="B122" s="15"/>
+      <c r="C122" s="18"/>
+      <c r="D122" s="16"/>
+      <c r="E122" s="15"/>
     </row>
     <row r="123" spans="1:5">
-      <c r="A123" s="5"/>
-      <c r="B123" s="5"/>
-      <c r="C123" s="13"/>
-      <c r="D123" s="12"/>
-      <c r="E123" s="5"/>
+      <c r="A123" s="15"/>
+      <c r="B123" s="15"/>
+      <c r="C123" s="18"/>
+      <c r="D123" s="16"/>
+      <c r="E123" s="15"/>
     </row>
     <row r="124" spans="1:5">
-      <c r="A124" s="5"/>
-      <c r="B124" s="5"/>
-      <c r="C124" s="13"/>
-      <c r="D124" s="12"/>
-      <c r="E124" s="5"/>
+      <c r="A124" s="15"/>
+      <c r="B124" s="15"/>
+      <c r="C124" s="18"/>
+      <c r="D124" s="16"/>
+      <c r="E124" s="15"/>
     </row>
     <row r="125" spans="1:5">
-      <c r="A125" s="5"/>
-      <c r="B125" s="5"/>
-      <c r="C125" s="13"/>
-      <c r="D125" s="12"/>
-      <c r="E125" s="5"/>
+      <c r="A125" s="15"/>
+      <c r="B125" s="15"/>
+      <c r="C125" s="18"/>
+      <c r="D125" s="16"/>
+      <c r="E125" s="15"/>
     </row>
     <row r="126" spans="1:5">
-      <c r="A126" s="5"/>
-      <c r="B126" s="5"/>
-      <c r="C126" s="15"/>
-      <c r="D126" s="12"/>
-      <c r="E126" s="5"/>
+      <c r="A126" s="15"/>
+      <c r="B126" s="15"/>
+      <c r="C126" s="19"/>
+      <c r="D126" s="16"/>
+      <c r="E126" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3211,7 +3316,7 @@
   <cols>
     <col min="1" max="1" width="8.72727272727273" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.72727272727273" style="2" customWidth="1"/>
-    <col min="3" max="3" width="33.3636363636364" style="1" customWidth="1"/>
+    <col min="3" max="3" width="47.6363636363636" style="1" customWidth="1"/>
     <col min="4" max="4" width="255.636363636364" style="1" customWidth="1"/>
     <col min="5" max="5" width="20.2727272727273" style="1" customWidth="1"/>
     <col min="6" max="6" width="9.72727272727273" style="1" customWidth="1"/>
@@ -3229,13 +3334,13 @@
         <v>34</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -3250,7 +3355,7 @@
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F2" s="5"/>
     </row>
@@ -3264,7 +3369,7 @@
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F3" s="5"/>
     </row>
@@ -3277,10 +3382,10 @@
         <v>37</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F4" s="5"/>
     </row>
@@ -3293,10 +3398,10 @@
         <v>37</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F5" s="5"/>
     </row>
@@ -3312,7 +3417,7 @@
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F6" s="5"/>
     </row>
@@ -3326,7 +3431,7 @@
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F7" s="5"/>
     </row>
@@ -3339,10 +3444,10 @@
         <v>39</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F8" s="5"/>
     </row>
@@ -3355,10 +3460,10 @@
         <v>39</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F9" s="5"/>
     </row>
@@ -3374,7 +3479,7 @@
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F10" s="5"/>
     </row>
@@ -3388,7 +3493,7 @@
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F11" s="5"/>
     </row>
@@ -3401,10 +3506,10 @@
         <v>41</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F12" s="5"/>
     </row>
@@ -3417,10 +3522,10 @@
         <v>41</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F13" s="5"/>
     </row>
@@ -3436,7 +3541,7 @@
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F14" s="5"/>
     </row>
@@ -3450,7 +3555,7 @@
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F15" s="5"/>
     </row>
@@ -3463,10 +3568,10 @@
         <v>43</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F16" s="5"/>
     </row>
@@ -3479,10 +3584,10 @@
         <v>43</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F17" s="5"/>
     </row>
@@ -3498,7 +3603,7 @@
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F18" s="5"/>
     </row>
@@ -3512,7 +3617,7 @@
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F19" s="5"/>
     </row>
@@ -3525,10 +3630,10 @@
         <v>45</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F20" s="5"/>
     </row>
@@ -3541,10 +3646,10 @@
         <v>45</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F21" s="5"/>
     </row>
@@ -3560,7 +3665,7 @@
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F22" s="5"/>
     </row>
@@ -3574,7 +3679,7 @@
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F23" s="5"/>
     </row>
@@ -3587,10 +3692,10 @@
         <v>47</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F24" s="5"/>
     </row>
@@ -3603,10 +3708,10 @@
         <v>47</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F25" s="5"/>
     </row>
@@ -3622,7 +3727,7 @@
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F26" s="5"/>
     </row>
@@ -3636,7 +3741,7 @@
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F27" s="5"/>
     </row>
@@ -3649,10 +3754,10 @@
         <v>49</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F28" s="5"/>
     </row>
@@ -3665,10 +3770,10 @@
         <v>49</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F29" s="5"/>
     </row>
@@ -3684,7 +3789,7 @@
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F30" s="5"/>
     </row>
@@ -3698,7 +3803,7 @@
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F31" s="5"/>
     </row>
@@ -3711,10 +3816,10 @@
         <v>51</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F32" s="5"/>
     </row>
@@ -3727,10 +3832,10 @@
         <v>51</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F33" s="5"/>
     </row>
@@ -3746,7 +3851,7 @@
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F34" s="5"/>
     </row>
@@ -3760,7 +3865,7 @@
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F35" s="5"/>
     </row>
@@ -3773,10 +3878,10 @@
         <v>53</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F36" s="5"/>
     </row>
@@ -3789,10 +3894,10 @@
         <v>53</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F37" s="5"/>
     </row>
@@ -3808,7 +3913,7 @@
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F38" s="5"/>
     </row>
@@ -3822,7 +3927,7 @@
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F39" s="5"/>
     </row>
@@ -3835,10 +3940,10 @@
         <v>55</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F40" s="5"/>
     </row>
@@ -3851,10 +3956,10 @@
         <v>55</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F41" s="5"/>
     </row>
@@ -3870,7 +3975,7 @@
       </c>
       <c r="D42" s="6"/>
       <c r="E42" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F42" s="5"/>
     </row>
@@ -3884,7 +3989,7 @@
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F43" s="5"/>
     </row>
@@ -3897,10 +4002,10 @@
         <v>57</v>
       </c>
       <c r="D44" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="E44" s="5" t="s">
         <v>129</v>
-      </c>
-      <c r="E44" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="F44" s="5"/>
     </row>
@@ -3913,10 +4018,10 @@
         <v>57</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F45" s="5"/>
     </row>
@@ -3932,7 +4037,7 @@
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F46" s="5"/>
     </row>
@@ -3946,7 +4051,7 @@
       </c>
       <c r="D47" s="6"/>
       <c r="E47" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F47" s="5"/>
     </row>
@@ -3959,10 +4064,10 @@
         <v>59</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F48" s="5"/>
     </row>
@@ -3975,10 +4080,10 @@
         <v>59</v>
       </c>
       <c r="D49" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="E49" s="5" t="s">
         <v>130</v>
-      </c>
-      <c r="E49" s="5" t="s">
-        <v>119</v>
       </c>
       <c r="F49" s="5"/>
     </row>
@@ -3994,7 +4099,7 @@
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F50" s="5"/>
     </row>
@@ -4008,7 +4113,7 @@
       </c>
       <c r="D51" s="6"/>
       <c r="E51" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F51" s="5"/>
     </row>
@@ -4021,10 +4126,10 @@
         <v>61</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F52" s="5"/>
     </row>
@@ -4037,10 +4142,10 @@
         <v>61</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F53" s="5"/>
     </row>
@@ -4056,7 +4161,7 @@
       </c>
       <c r="D54" s="6"/>
       <c r="E54" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F54" s="5"/>
     </row>
@@ -4070,7 +4175,7 @@
       </c>
       <c r="D55" s="6"/>
       <c r="E55" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F55" s="5"/>
     </row>
@@ -4083,10 +4188,10 @@
         <v>63</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F56" s="5"/>
     </row>
@@ -4099,10 +4204,10 @@
         <v>63</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F57" s="5"/>
     </row>
@@ -4118,7 +4223,7 @@
       </c>
       <c r="D58" s="6"/>
       <c r="E58" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F58" s="5"/>
     </row>
@@ -4132,7 +4237,7 @@
       </c>
       <c r="D59" s="6"/>
       <c r="E59" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F59" s="5"/>
     </row>
@@ -4145,10 +4250,10 @@
         <v>65</v>
       </c>
       <c r="D60" s="11" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F60" s="5"/>
     </row>
@@ -4161,10 +4266,10 @@
         <v>65</v>
       </c>
       <c r="D61" s="11" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F61" s="5"/>
     </row>
@@ -4180,7 +4285,7 @@
       </c>
       <c r="D62" s="6"/>
       <c r="E62" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F62" s="5"/>
     </row>
@@ -4194,7 +4299,7 @@
       </c>
       <c r="D63" s="6"/>
       <c r="E63" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F63" s="5"/>
     </row>
@@ -4207,10 +4312,10 @@
         <v>67</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F64" s="5"/>
     </row>
@@ -4223,10 +4328,10 @@
         <v>67</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F65" s="5"/>
     </row>
@@ -4242,7 +4347,7 @@
       </c>
       <c r="D66" s="6"/>
       <c r="E66" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F66" s="5"/>
     </row>
@@ -4256,7 +4361,7 @@
       </c>
       <c r="D67" s="6"/>
       <c r="E67" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F67" s="5"/>
     </row>
@@ -4269,10 +4374,10 @@
         <v>69</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F68" s="5"/>
     </row>
@@ -4285,10 +4390,10 @@
         <v>69</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F69" s="5"/>
     </row>
@@ -4304,7 +4409,7 @@
       </c>
       <c r="D70" s="6"/>
       <c r="E70" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F70" s="5"/>
     </row>
@@ -4318,7 +4423,7 @@
       </c>
       <c r="D71" s="6"/>
       <c r="E71" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F71" s="5"/>
     </row>
@@ -4331,10 +4436,10 @@
         <v>71</v>
       </c>
       <c r="D72" s="11" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F72" s="5"/>
     </row>
@@ -4347,10 +4452,10 @@
         <v>71</v>
       </c>
       <c r="D73" s="11" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F73" s="5"/>
     </row>
@@ -4366,7 +4471,7 @@
       </c>
       <c r="D74" s="6"/>
       <c r="E74" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F74" s="5"/>
     </row>
@@ -4380,7 +4485,7 @@
       </c>
       <c r="D75" s="6"/>
       <c r="E75" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F75" s="5"/>
     </row>
@@ -4393,10 +4498,10 @@
         <v>73</v>
       </c>
       <c r="D76" s="11" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F76" s="5"/>
     </row>
@@ -4409,10 +4514,10 @@
         <v>73</v>
       </c>
       <c r="D77" s="11" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F77" s="5"/>
     </row>
@@ -4428,7 +4533,7 @@
       </c>
       <c r="D78" s="6"/>
       <c r="E78" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F78" s="5"/>
     </row>
@@ -4442,7 +4547,7 @@
       </c>
       <c r="D79" s="6"/>
       <c r="E79" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F79" s="5"/>
     </row>
@@ -4455,10 +4560,10 @@
         <v>75</v>
       </c>
       <c r="D80" s="11" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F80" s="5"/>
     </row>
@@ -4471,10 +4576,10 @@
         <v>75</v>
       </c>
       <c r="D81" s="11" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F81" s="5"/>
     </row>
@@ -4490,7 +4595,7 @@
       </c>
       <c r="D82" s="6"/>
       <c r="E82" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F82" s="5"/>
     </row>
@@ -4504,7 +4609,7 @@
       </c>
       <c r="D83" s="6"/>
       <c r="E83" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F83" s="5"/>
     </row>
@@ -4517,10 +4622,10 @@
         <v>77</v>
       </c>
       <c r="D84" s="11" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F84" s="5"/>
     </row>
@@ -4533,10 +4638,10 @@
         <v>77</v>
       </c>
       <c r="D85" s="11" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F85" s="5"/>
     </row>
@@ -4552,7 +4657,7 @@
       </c>
       <c r="D86" s="6"/>
       <c r="E86" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F86" s="5"/>
     </row>
@@ -4566,7 +4671,7 @@
       </c>
       <c r="D87" s="6"/>
       <c r="E87" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F87" s="5"/>
     </row>
@@ -4579,10 +4684,10 @@
         <v>79</v>
       </c>
       <c r="D88" s="11" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F88" s="5"/>
     </row>
@@ -4595,10 +4700,10 @@
         <v>79</v>
       </c>
       <c r="D89" s="11" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F89" s="5"/>
     </row>
@@ -4614,7 +4719,7 @@
       </c>
       <c r="D90" s="6"/>
       <c r="E90" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F90" s="5"/>
     </row>
@@ -4628,7 +4733,7 @@
       </c>
       <c r="D91" s="6"/>
       <c r="E91" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F91" s="5"/>
     </row>
@@ -4641,10 +4746,10 @@
         <v>81</v>
       </c>
       <c r="D92" s="11" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F92" s="5"/>
     </row>
@@ -4657,10 +4762,10 @@
         <v>81</v>
       </c>
       <c r="D93" s="11" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F93" s="5"/>
     </row>
@@ -4676,7 +4781,7 @@
       </c>
       <c r="D94" s="6"/>
       <c r="E94" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F94" s="5"/>
     </row>
@@ -4690,7 +4795,7 @@
       </c>
       <c r="D95" s="6"/>
       <c r="E95" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F95" s="5"/>
     </row>
@@ -4703,10 +4808,10 @@
         <v>83</v>
       </c>
       <c r="D96" s="11" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F96" s="5"/>
     </row>
@@ -4719,10 +4824,10 @@
         <v>83</v>
       </c>
       <c r="D97" s="11" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F97" s="5"/>
     </row>
@@ -4738,7 +4843,7 @@
       </c>
       <c r="D98" s="6"/>
       <c r="E98" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F98" s="5"/>
     </row>
@@ -4752,7 +4857,7 @@
       </c>
       <c r="D99" s="6"/>
       <c r="E99" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F99" s="5"/>
     </row>
@@ -4765,10 +4870,10 @@
         <v>85</v>
       </c>
       <c r="D100" s="11" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F100" s="5"/>
     </row>
@@ -4781,10 +4886,10 @@
         <v>85</v>
       </c>
       <c r="D101" s="11" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="E101" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F101" s="5"/>
     </row>
@@ -4800,7 +4905,7 @@
       </c>
       <c r="D102" s="6"/>
       <c r="E102" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F102" s="5"/>
     </row>
@@ -4814,7 +4919,7 @@
       </c>
       <c r="D103" s="6"/>
       <c r="E103" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F103" s="5"/>
     </row>
@@ -4827,10 +4932,10 @@
         <v>87</v>
       </c>
       <c r="D104" s="11" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F104" s="5"/>
     </row>
@@ -4843,10 +4948,10 @@
         <v>87</v>
       </c>
       <c r="D105" s="11" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F105" s="5"/>
     </row>
@@ -4862,7 +4967,7 @@
       </c>
       <c r="D106" s="6"/>
       <c r="E106" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F106" s="5"/>
     </row>
@@ -4876,7 +4981,7 @@
       </c>
       <c r="D107" s="6"/>
       <c r="E107" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F107" s="5"/>
     </row>
@@ -4889,10 +4994,10 @@
         <v>89</v>
       </c>
       <c r="D108" s="11" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F108" s="5"/>
     </row>
@@ -4905,10 +5010,10 @@
         <v>89</v>
       </c>
       <c r="D109" s="11" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="E109" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F109" s="5"/>
     </row>
@@ -4924,7 +5029,7 @@
       </c>
       <c r="D110" s="6"/>
       <c r="E110" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F110" s="5"/>
     </row>
@@ -4938,7 +5043,7 @@
       </c>
       <c r="D111" s="6"/>
       <c r="E111" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F111" s="5"/>
     </row>
@@ -4951,10 +5056,10 @@
         <v>91</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F112" s="5"/>
     </row>
@@ -4967,10 +5072,10 @@
         <v>91</v>
       </c>
       <c r="D113" s="6" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="E113" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F113" s="5"/>
     </row>
@@ -4986,7 +5091,7 @@
       </c>
       <c r="D114" s="6"/>
       <c r="E114" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F114" s="5"/>
     </row>
@@ -5000,7 +5105,7 @@
       </c>
       <c r="D115" s="6"/>
       <c r="E115" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F115" s="5"/>
     </row>
@@ -5013,10 +5118,10 @@
         <v>93</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F116" s="5"/>
     </row>
@@ -5029,10 +5134,10 @@
         <v>93</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="E117" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F117" s="5"/>
     </row>
@@ -5048,7 +5153,7 @@
       </c>
       <c r="D118" s="6"/>
       <c r="E118" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F118" s="5"/>
     </row>
@@ -5062,7 +5167,7 @@
       </c>
       <c r="D119" s="6"/>
       <c r="E119" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F119" s="5"/>
     </row>
@@ -5075,10 +5180,10 @@
         <v>95</v>
       </c>
       <c r="D120" s="6" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F120" s="5"/>
     </row>
@@ -5091,10 +5196,10 @@
         <v>95</v>
       </c>
       <c r="D121" s="6" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="E121" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F121" s="5"/>
     </row>
@@ -5110,7 +5215,7 @@
       </c>
       <c r="D122" s="6"/>
       <c r="E122" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F122" s="5"/>
     </row>
@@ -5124,7 +5229,7 @@
       </c>
       <c r="D123" s="6"/>
       <c r="E123" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F123" s="5"/>
     </row>
@@ -5137,10 +5242,10 @@
         <v>97</v>
       </c>
       <c r="D124" s="6" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="E124" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F124" s="5"/>
     </row>
@@ -5153,10 +5258,10 @@
         <v>97</v>
       </c>
       <c r="D125" s="6" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="E125" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F125" s="5"/>
     </row>
@@ -5172,7 +5277,7 @@
       </c>
       <c r="D126" s="6"/>
       <c r="E126" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F126" s="5"/>
     </row>
@@ -5186,7 +5291,7 @@
       </c>
       <c r="D127" s="6"/>
       <c r="E127" s="5" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="F127" s="5"/>
     </row>
@@ -5199,10 +5304,10 @@
         <v>99</v>
       </c>
       <c r="D128" s="6" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="E128" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="F128" s="5"/>
     </row>
@@ -5215,10 +5320,10 @@
         <v>99</v>
       </c>
       <c r="D129" s="6" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="E129" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F129" s="5"/>
     </row>

</xml_diff>

<commit_message>
changes made to sql scripts
</commit_message>
<xml_diff>
--- a/silver_layer_data_validation_databrick_catalog/queries/validation_queries.xlsx
+++ b/silver_layer_data_validation_databrick_catalog/queries/validation_queries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6080" activeTab="2"/>
+    <workbookView windowWidth="19200" windowHeight="6800" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="db" sheetId="1" r:id="rId1"/>
@@ -146,175 +146,175 @@
     <t>amendment_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\amendment_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\amendment_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>application_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\application_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\application_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>application_support_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\application_support_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\application_support_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>assessment_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\assessment_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\assessment_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>certification_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\certification_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\certification_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>customer_enterprise_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\customer_enterprise_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\customer_enterprise_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>customer_individual_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\customer_individual_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\customer_individual_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>employee_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\employee_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\employee_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>financing_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\financing_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\financing_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>iban_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\iban_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\iban_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>moic_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\moic_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\moic_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>payment_assessment_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\payment_assessment_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\payment_assessment_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>payment_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\payment_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\payment_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>payment_plan_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\payment_plan_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\payment_plan_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>payment_support_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\payment_support_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\payment_support_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>product_services_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\product_services_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\product_services_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>program_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\program_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\program_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>sector_isic_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\sector_isic_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\sector_isic_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>security_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\security_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\security_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>service_fee_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\service_fee_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\service_fee_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>special_condition_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\special_condition_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\special_condition_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>support_structure_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\support_structure_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\support_structure_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>ticket_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\ticket_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\ticket_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>training_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\training_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\training_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>unstructured_questions_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\unstructured_questions_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\unstructured_questions_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>user_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\user_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\user_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>wage_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\wage_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\wage_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>workflow_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\workflow_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\workflow_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>withdrawal_base</t>
   </si>
   <si>
-    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\withdrawal_base.sql</t>
+    <t>C:\Users\MODICHERLA\OneDrive - Hexalytics, Inc\Documents\databricks_project\silver_layer_data_validation_databrick_catalog\queries\sql_union_all_sources\withdrawal_base_compare_bronze_silver.sql</t>
   </si>
   <si>
     <t>infor_special_project_compare_bronze_silver</t>
@@ -509,7 +509,7 @@
     <t>source_system_name,process_id,id_withdraw,withdraw_ref</t>
   </si>
   <si>
-    <t>source_system_name,program_id,dimension_code,accounting_unit_code</t>
+    <t>source_system_name,contract_id,contract_description,commitment_amount_remaining,vendor_reference,maximum_amount,primary_contact,contract_name,accounting_unit_code,contract_status,is_on_hold,performance_bond_pct,vendor_name,vendor_id,expiration_date,contract_type,effective_date</t>
   </si>
   <si>
     <t>source_system_name,meeting_subject,start_datetime,end_datetime,company_name,created_on</t>
@@ -1221,7 +1221,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1261,9 +1261,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1840,31 +1837,31 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:9">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="22" t="s">
+      <c r="B1" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="E1" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="22" t="s">
+      <c r="G1" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="22" t="s">
+      <c r="H1" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="22" t="s">
+      <c r="I1" s="21" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1884,10 +1881,10 @@
       <c r="E2" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="23" t="s">
+      <c r="F2" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="24" t="s">
+      <c r="G2" s="23" t="s">
         <v>14</v>
       </c>
       <c r="H2" s="13" t="b">
@@ -1913,10 +1910,10 @@
       <c r="E3" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="G3" s="23" t="s">
         <v>17</v>
       </c>
       <c r="H3" s="13" t="b">
@@ -1942,10 +1939,10 @@
       <c r="E4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="24" t="s">
+      <c r="G4" s="23" t="s">
         <v>21</v>
       </c>
       <c r="H4" s="13" t="b">
@@ -1971,10 +1968,10 @@
       <c r="E5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="24" t="s">
+      <c r="G5" s="23" t="s">
         <v>22</v>
       </c>
       <c r="H5" s="13" t="b">
@@ -1996,25 +1993,25 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="4"/>
   <cols>
-    <col min="3" max="3" width="12.6363636363636" style="20" customWidth="1"/>
-    <col min="4" max="4" width="46.4545454545455" style="20" customWidth="1"/>
-    <col min="5" max="5" width="44.8181818181818" style="20" customWidth="1"/>
+    <col min="3" max="3" width="12.6363636363636" style="19" customWidth="1"/>
+    <col min="4" max="4" width="46.4545454545455" style="19" customWidth="1"/>
+    <col min="5" max="5" width="44.8181818181818" style="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="20" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2092,7 +2089,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>37</v>
@@ -2107,7 +2104,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>39</v>
@@ -2137,7 +2134,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>43</v>
@@ -2212,7 +2209,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>53</v>
@@ -2302,7 +2299,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" s="14" t="s">
         <v>65</v>
@@ -2347,7 +2344,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C19" s="14" t="s">
         <v>71</v>
@@ -2437,7 +2434,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C25" s="14" t="s">
         <v>83</v>
@@ -2732,575 +2729,329 @@
       </c>
       <c r="E44" s="5"/>
     </row>
-    <row r="45" s="12" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A45" s="15"/>
-      <c r="B45" s="15"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="15"/>
-    </row>
-    <row r="46" s="12" customFormat="1" ht="29" customHeight="1" spans="1:5">
-      <c r="A46" s="15"/>
-      <c r="B46" s="15"/>
-      <c r="D46" s="16"/>
-      <c r="E46" s="15"/>
-    </row>
-    <row r="47" s="12" customFormat="1" ht="34" customHeight="1" spans="1:5">
-      <c r="A47" s="15"/>
-      <c r="B47" s="15"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="15"/>
-    </row>
-    <row r="48" s="12" customFormat="1" ht="31" customHeight="1" spans="1:5">
-      <c r="A48" s="15"/>
-      <c r="B48" s="15"/>
-      <c r="D48" s="16"/>
-      <c r="E48" s="15"/>
-    </row>
-    <row r="49" s="12" customFormat="1" ht="36" customHeight="1" spans="1:5">
-      <c r="A49" s="15"/>
-      <c r="B49" s="15"/>
-      <c r="C49" s="17"/>
-      <c r="D49" s="16"/>
-      <c r="E49" s="15"/>
-    </row>
-    <row r="50" s="12" customFormat="1" ht="31" customHeight="1" spans="1:5">
-      <c r="A50" s="15"/>
-      <c r="B50" s="15"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="16"/>
-      <c r="E50" s="15"/>
-    </row>
-    <row r="51" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A51" s="15"/>
-      <c r="B51" s="15"/>
-      <c r="C51" s="18"/>
-      <c r="D51" s="16"/>
-      <c r="E51" s="15"/>
-    </row>
-    <row r="52" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A52" s="15"/>
-      <c r="B52" s="15"/>
-      <c r="C52" s="18"/>
-      <c r="D52" s="16"/>
-      <c r="E52" s="15"/>
-    </row>
-    <row r="53" s="12" customFormat="1" ht="27" customHeight="1" spans="1:5">
-      <c r="A53" s="15"/>
-      <c r="B53" s="15"/>
-      <c r="C53" s="18"/>
-      <c r="D53" s="16"/>
-      <c r="E53" s="15"/>
-    </row>
-    <row r="54" s="12" customFormat="1" ht="31" customHeight="1" spans="1:5">
-      <c r="A54" s="15"/>
-      <c r="B54" s="15"/>
-      <c r="C54" s="18"/>
-      <c r="D54" s="16"/>
-      <c r="E54" s="15"/>
-    </row>
-    <row r="55" s="12" customFormat="1" ht="36" customHeight="1" spans="1:5">
-      <c r="A55" s="15"/>
-      <c r="B55" s="15"/>
-      <c r="C55" s="18"/>
-      <c r="D55" s="16"/>
-      <c r="E55" s="15"/>
-    </row>
-    <row r="56" s="12" customFormat="1" spans="1:5">
-      <c r="A56" s="15"/>
-      <c r="B56" s="15"/>
-      <c r="C56" s="18"/>
-      <c r="D56" s="16"/>
-      <c r="E56" s="15"/>
-    </row>
-    <row r="57" s="12" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A57" s="15"/>
-      <c r="B57" s="15"/>
-      <c r="C57" s="18"/>
-      <c r="D57" s="16"/>
-      <c r="E57" s="15"/>
-    </row>
-    <row r="58" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A58" s="15"/>
-      <c r="B58" s="15"/>
-      <c r="C58" s="18"/>
-      <c r="D58" s="16"/>
-      <c r="E58" s="15"/>
-    </row>
-    <row r="59" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A59" s="15"/>
-      <c r="B59" s="15"/>
-      <c r="C59" s="18"/>
-      <c r="D59" s="16"/>
-      <c r="E59" s="15"/>
-    </row>
-    <row r="60" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A60" s="15"/>
-      <c r="B60" s="15"/>
-      <c r="C60" s="18"/>
-      <c r="D60" s="16"/>
-      <c r="E60" s="15"/>
-    </row>
-    <row r="61" s="12" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A61" s="15"/>
-      <c r="B61" s="15"/>
-      <c r="C61" s="18"/>
-      <c r="D61" s="16"/>
-      <c r="E61" s="15"/>
-    </row>
-    <row r="62" s="12" customFormat="1" ht="29" customHeight="1" spans="1:5">
-      <c r="A62" s="15"/>
-      <c r="B62" s="15"/>
-      <c r="C62" s="18"/>
-      <c r="D62" s="16"/>
-      <c r="E62" s="15"/>
-    </row>
-    <row r="63" s="12" customFormat="1" ht="30" customHeight="1" spans="1:5">
-      <c r="A63" s="15"/>
-      <c r="B63" s="15"/>
-      <c r="C63" s="18"/>
-      <c r="D63" s="16"/>
-      <c r="E63" s="15"/>
-    </row>
-    <row r="64" s="12" customFormat="1" ht="29" customHeight="1" spans="1:5">
-      <c r="A64" s="15"/>
-      <c r="B64" s="15"/>
-      <c r="C64" s="18"/>
-      <c r="D64" s="16"/>
-      <c r="E64" s="15"/>
-    </row>
-    <row r="65" s="12" customFormat="1" ht="31" customHeight="1" spans="1:5">
-      <c r="A65" s="15"/>
-      <c r="B65" s="15"/>
-      <c r="C65" s="18"/>
-      <c r="D65" s="16"/>
-      <c r="E65" s="15"/>
-    </row>
-    <row r="66" s="12" customFormat="1" ht="30" customHeight="1" spans="1:5">
-      <c r="A66" s="15"/>
-      <c r="B66" s="15"/>
-      <c r="C66" s="18"/>
-      <c r="D66" s="16"/>
-      <c r="E66" s="15"/>
-    </row>
-    <row r="67" s="12" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A67" s="15"/>
-      <c r="B67" s="15"/>
-      <c r="C67" s="18"/>
-      <c r="D67" s="16"/>
-      <c r="E67" s="15"/>
-    </row>
-    <row r="68" s="12" customFormat="1" ht="33" customHeight="1" spans="1:5">
-      <c r="A68" s="15"/>
-      <c r="B68" s="15"/>
-      <c r="C68" s="18"/>
-      <c r="D68" s="16"/>
-      <c r="E68" s="15"/>
-    </row>
-    <row r="69" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A69" s="15"/>
-      <c r="B69" s="15"/>
-      <c r="C69" s="18"/>
-      <c r="D69" s="16"/>
-      <c r="E69" s="15"/>
-    </row>
-    <row r="70" s="12" customFormat="1" ht="32" customHeight="1" spans="1:5">
-      <c r="A70" s="15"/>
-      <c r="B70" s="15"/>
-      <c r="C70" s="18"/>
-      <c r="D70" s="16"/>
-      <c r="E70" s="15"/>
-    </row>
-    <row r="71" s="12" customFormat="1" ht="31" customHeight="1" spans="1:5">
-      <c r="A71" s="15"/>
-      <c r="B71" s="15"/>
-      <c r="C71" s="18"/>
-      <c r="D71" s="16"/>
-      <c r="E71" s="15"/>
-    </row>
-    <row r="72" s="12" customFormat="1" spans="1:5">
-      <c r="A72" s="15"/>
-      <c r="B72" s="15"/>
-      <c r="C72" s="18"/>
-      <c r="D72" s="16"/>
-      <c r="E72" s="15"/>
-    </row>
-    <row r="73" s="12" customFormat="1" spans="1:5">
-      <c r="A73" s="15"/>
-      <c r="B73" s="15"/>
-      <c r="C73" s="18"/>
-      <c r="D73" s="16"/>
-      <c r="E73" s="15"/>
-    </row>
-    <row r="74" s="12" customFormat="1" spans="1:5">
-      <c r="A74" s="15"/>
-      <c r="B74" s="15"/>
-      <c r="C74" s="18"/>
-      <c r="D74" s="16"/>
-      <c r="E74" s="15"/>
-    </row>
-    <row r="75" s="12" customFormat="1" spans="1:5">
-      <c r="A75" s="15"/>
-      <c r="B75" s="15"/>
-      <c r="C75" s="18"/>
-      <c r="D75" s="16"/>
-      <c r="E75" s="15"/>
-    </row>
-    <row r="76" s="12" customFormat="1" spans="1:5">
-      <c r="A76" s="15"/>
-      <c r="B76" s="15"/>
-      <c r="C76" s="18"/>
-      <c r="D76" s="16"/>
-      <c r="E76" s="15"/>
-    </row>
-    <row r="77" s="12" customFormat="1" spans="1:5">
-      <c r="A77" s="15"/>
-      <c r="B77" s="15"/>
-      <c r="C77" s="18"/>
-      <c r="D77" s="16"/>
-      <c r="E77" s="15"/>
-    </row>
-    <row r="78" spans="1:5">
-      <c r="A78" s="15"/>
-      <c r="B78" s="15"/>
-      <c r="C78" s="18"/>
-      <c r="D78" s="16"/>
-      <c r="E78" s="15"/>
-    </row>
-    <row r="79" spans="1:5">
-      <c r="A79" s="15"/>
-      <c r="B79" s="15"/>
-      <c r="C79" s="18"/>
-      <c r="D79" s="16"/>
-      <c r="E79" s="15"/>
-    </row>
-    <row r="80" spans="1:5">
-      <c r="A80" s="15"/>
-      <c r="B80" s="15"/>
-      <c r="C80" s="18"/>
-      <c r="D80" s="16"/>
-      <c r="E80" s="15"/>
-    </row>
-    <row r="81" spans="1:5">
-      <c r="A81" s="15"/>
-      <c r="B81" s="15"/>
-      <c r="C81" s="18"/>
-      <c r="D81" s="16"/>
-      <c r="E81" s="15"/>
-    </row>
-    <row r="82" spans="1:5">
-      <c r="A82" s="15"/>
-      <c r="B82" s="15"/>
-      <c r="C82" s="18"/>
-      <c r="D82" s="16"/>
-      <c r="E82" s="15"/>
-    </row>
-    <row r="83" spans="1:5">
-      <c r="A83" s="15"/>
-      <c r="B83" s="15"/>
-      <c r="C83" s="18"/>
-      <c r="D83" s="16"/>
-      <c r="E83" s="15"/>
-    </row>
-    <row r="84" spans="1:5">
-      <c r="A84" s="15"/>
-      <c r="B84" s="15"/>
-      <c r="C84" s="18"/>
-      <c r="D84" s="16"/>
-      <c r="E84" s="15"/>
-    </row>
-    <row r="85" spans="1:5">
-      <c r="A85" s="15"/>
-      <c r="B85" s="15"/>
-      <c r="C85" s="18"/>
-      <c r="D85" s="16"/>
-      <c r="E85" s="15"/>
-    </row>
-    <row r="86" spans="1:5">
-      <c r="A86" s="15"/>
-      <c r="B86" s="15"/>
-      <c r="C86" s="18"/>
-      <c r="D86" s="16"/>
-      <c r="E86" s="15"/>
-    </row>
-    <row r="87" spans="1:5">
-      <c r="A87" s="15"/>
-      <c r="B87" s="15"/>
-      <c r="C87" s="18"/>
-      <c r="D87" s="16"/>
-      <c r="E87" s="15"/>
-    </row>
-    <row r="88" spans="1:5">
-      <c r="A88" s="15"/>
-      <c r="B88" s="15"/>
-      <c r="C88" s="18"/>
-      <c r="D88" s="16"/>
-      <c r="E88" s="15"/>
-    </row>
-    <row r="89" spans="1:5">
-      <c r="A89" s="15"/>
-      <c r="B89" s="15"/>
-      <c r="C89" s="18"/>
-      <c r="D89" s="16"/>
-      <c r="E89" s="15"/>
-    </row>
-    <row r="90" spans="1:5">
-      <c r="A90" s="15"/>
-      <c r="B90" s="15"/>
-      <c r="C90" s="18"/>
-      <c r="D90" s="16"/>
-      <c r="E90" s="15"/>
-    </row>
-    <row r="91" spans="1:5">
-      <c r="A91" s="15"/>
-      <c r="B91" s="15"/>
-      <c r="C91" s="18"/>
-      <c r="D91" s="16"/>
-      <c r="E91" s="15"/>
-    </row>
-    <row r="92" spans="1:5">
-      <c r="A92" s="15"/>
-      <c r="B92" s="15"/>
-      <c r="C92" s="18"/>
-      <c r="D92" s="16"/>
-      <c r="E92" s="15"/>
-    </row>
-    <row r="93" spans="1:5">
-      <c r="A93" s="15"/>
-      <c r="B93" s="15"/>
-      <c r="C93" s="18"/>
-      <c r="D93" s="16"/>
-      <c r="E93" s="15"/>
-    </row>
-    <row r="94" spans="1:5">
-      <c r="A94" s="15"/>
-      <c r="B94" s="15"/>
-      <c r="C94" s="18"/>
-      <c r="D94" s="16"/>
-      <c r="E94" s="15"/>
-    </row>
-    <row r="95" spans="1:5">
-      <c r="A95" s="15"/>
-      <c r="B95" s="15"/>
-      <c r="C95" s="18"/>
-      <c r="D95" s="16"/>
-      <c r="E95" s="15"/>
-    </row>
-    <row r="96" spans="1:5">
-      <c r="A96" s="15"/>
-      <c r="B96" s="15"/>
-      <c r="C96" s="18"/>
-      <c r="D96" s="16"/>
-      <c r="E96" s="15"/>
-    </row>
-    <row r="97" spans="1:5">
-      <c r="A97" s="15"/>
-      <c r="B97" s="15"/>
-      <c r="C97" s="18"/>
-      <c r="D97" s="16"/>
-      <c r="E97" s="15"/>
-    </row>
-    <row r="98" spans="1:5">
-      <c r="A98" s="15"/>
-      <c r="B98" s="15"/>
-      <c r="C98" s="18"/>
-      <c r="D98" s="16"/>
-      <c r="E98" s="15"/>
-    </row>
-    <row r="99" spans="1:5">
-      <c r="A99" s="15"/>
-      <c r="B99" s="15"/>
-      <c r="C99" s="18"/>
-      <c r="D99" s="16"/>
-      <c r="E99" s="15"/>
-    </row>
-    <row r="100" spans="1:5">
-      <c r="A100" s="15"/>
-      <c r="B100" s="15"/>
-      <c r="C100" s="18"/>
-      <c r="D100" s="16"/>
-      <c r="E100" s="15"/>
-    </row>
-    <row r="101" spans="1:5">
-      <c r="A101" s="15"/>
-      <c r="B101" s="15"/>
-      <c r="C101" s="18"/>
-      <c r="D101" s="16"/>
-      <c r="E101" s="15"/>
-    </row>
-    <row r="102" spans="1:5">
-      <c r="A102" s="15"/>
-      <c r="B102" s="15"/>
-      <c r="C102" s="18"/>
-      <c r="D102" s="16"/>
-      <c r="E102" s="15"/>
-    </row>
-    <row r="103" spans="1:5">
-      <c r="A103" s="15"/>
-      <c r="B103" s="15"/>
-      <c r="C103" s="18"/>
-      <c r="D103" s="16"/>
-      <c r="E103" s="15"/>
-    </row>
-    <row r="104" spans="1:5">
-      <c r="A104" s="15"/>
-      <c r="B104" s="15"/>
-      <c r="C104" s="18"/>
-      <c r="D104" s="16"/>
-      <c r="E104" s="15"/>
-    </row>
-    <row r="105" spans="1:5">
-      <c r="A105" s="15"/>
-      <c r="B105" s="15"/>
-      <c r="C105" s="18"/>
-      <c r="D105" s="16"/>
-      <c r="E105" s="15"/>
-    </row>
-    <row r="106" spans="1:5">
-      <c r="A106" s="15"/>
-      <c r="B106" s="15"/>
-      <c r="C106" s="18"/>
-      <c r="D106" s="16"/>
-      <c r="E106" s="15"/>
-    </row>
-    <row r="107" spans="1:5">
-      <c r="A107" s="15"/>
-      <c r="B107" s="15"/>
-      <c r="C107" s="18"/>
-      <c r="D107" s="16"/>
-      <c r="E107" s="15"/>
-    </row>
-    <row r="108" spans="1:5">
-      <c r="A108" s="15"/>
-      <c r="B108" s="15"/>
-      <c r="C108" s="18"/>
-      <c r="D108" s="16"/>
-      <c r="E108" s="15"/>
-    </row>
-    <row r="109" spans="1:5">
-      <c r="A109" s="15"/>
-      <c r="B109" s="15"/>
-      <c r="C109" s="18"/>
-      <c r="D109" s="16"/>
-      <c r="E109" s="15"/>
-    </row>
-    <row r="110" spans="1:5">
-      <c r="A110" s="15"/>
-      <c r="B110" s="15"/>
-      <c r="C110" s="18"/>
-      <c r="D110" s="16"/>
-      <c r="E110" s="15"/>
-    </row>
-    <row r="111" spans="1:5">
-      <c r="A111" s="15"/>
-      <c r="B111" s="15"/>
-      <c r="C111" s="18"/>
-      <c r="D111" s="16"/>
-      <c r="E111" s="15"/>
-    </row>
-    <row r="112" spans="1:5">
-      <c r="A112" s="15"/>
-      <c r="B112" s="15"/>
-      <c r="C112" s="18"/>
-      <c r="D112" s="16"/>
-      <c r="E112" s="15"/>
-    </row>
-    <row r="113" spans="1:5">
-      <c r="A113" s="15"/>
-      <c r="B113" s="15"/>
-      <c r="C113" s="18"/>
-      <c r="D113" s="16"/>
-      <c r="E113" s="15"/>
-    </row>
-    <row r="114" spans="1:5">
-      <c r="A114" s="15"/>
-      <c r="B114" s="15"/>
-      <c r="C114" s="18"/>
-      <c r="D114" s="16"/>
-      <c r="E114" s="15"/>
-    </row>
-    <row r="115" spans="1:5">
-      <c r="A115" s="15"/>
-      <c r="B115" s="15"/>
-      <c r="C115" s="18"/>
-      <c r="D115" s="16"/>
-      <c r="E115" s="15"/>
-    </row>
-    <row r="116" spans="1:5">
-      <c r="A116" s="15"/>
-      <c r="B116" s="15"/>
-      <c r="C116" s="18"/>
-      <c r="D116" s="16"/>
-      <c r="E116" s="15"/>
-    </row>
-    <row r="117" spans="1:5">
-      <c r="A117" s="15"/>
-      <c r="B117" s="15"/>
-      <c r="C117" s="18"/>
-      <c r="D117" s="16"/>
-      <c r="E117" s="15"/>
-    </row>
-    <row r="118" spans="1:5">
-      <c r="A118" s="15"/>
-      <c r="B118" s="15"/>
-      <c r="C118" s="18"/>
-      <c r="D118" s="16"/>
-      <c r="E118" s="15"/>
-    </row>
-    <row r="119" spans="1:5">
-      <c r="A119" s="15"/>
-      <c r="B119" s="15"/>
-      <c r="C119" s="18"/>
-      <c r="D119" s="16"/>
-      <c r="E119" s="15"/>
-    </row>
-    <row r="120" spans="1:5">
-      <c r="A120" s="15"/>
-      <c r="B120" s="15"/>
-      <c r="C120" s="18"/>
-      <c r="D120" s="16"/>
-      <c r="E120" s="15"/>
-    </row>
-    <row r="121" spans="1:5">
-      <c r="A121" s="15"/>
-      <c r="B121" s="15"/>
-      <c r="C121" s="18"/>
-      <c r="D121" s="16"/>
-      <c r="E121" s="15"/>
-    </row>
-    <row r="122" spans="1:5">
-      <c r="A122" s="15"/>
-      <c r="B122" s="15"/>
-      <c r="C122" s="18"/>
-      <c r="D122" s="16"/>
-      <c r="E122" s="15"/>
-    </row>
-    <row r="123" spans="1:5">
-      <c r="A123" s="15"/>
-      <c r="B123" s="15"/>
-      <c r="C123" s="18"/>
-      <c r="D123" s="16"/>
-      <c r="E123" s="15"/>
-    </row>
-    <row r="124" spans="1:5">
-      <c r="A124" s="15"/>
-      <c r="B124" s="15"/>
-      <c r="C124" s="18"/>
-      <c r="D124" s="16"/>
-      <c r="E124" s="15"/>
-    </row>
-    <row r="125" spans="1:5">
-      <c r="A125" s="15"/>
-      <c r="B125" s="15"/>
-      <c r="C125" s="18"/>
-      <c r="D125" s="16"/>
-      <c r="E125" s="15"/>
-    </row>
-    <row r="126" spans="1:5">
-      <c r="A126" s="15"/>
-      <c r="B126" s="15"/>
-      <c r="C126" s="19"/>
-      <c r="D126" s="16"/>
-      <c r="E126" s="15"/>
+    <row r="45" s="12" customFormat="1" ht="33" customHeight="1" spans="4:4">
+      <c r="D45" s="15"/>
+    </row>
+    <row r="46" s="12" customFormat="1" ht="29" customHeight="1" spans="4:4">
+      <c r="D46" s="15"/>
+    </row>
+    <row r="47" s="12" customFormat="1" ht="34" customHeight="1" spans="4:4">
+      <c r="D47" s="15"/>
+    </row>
+    <row r="48" s="12" customFormat="1" ht="31" customHeight="1" spans="4:4">
+      <c r="D48" s="15"/>
+    </row>
+    <row r="49" s="12" customFormat="1" ht="36" customHeight="1" spans="3:4">
+      <c r="C49" s="16"/>
+      <c r="D49" s="15"/>
+    </row>
+    <row r="50" s="12" customFormat="1" ht="31" customHeight="1" spans="3:4">
+      <c r="C50" s="17"/>
+      <c r="D50" s="15"/>
+    </row>
+    <row r="51" s="12" customFormat="1" ht="32" customHeight="1" spans="3:4">
+      <c r="C51" s="17"/>
+      <c r="D51" s="15"/>
+    </row>
+    <row r="52" s="12" customFormat="1" ht="32" customHeight="1" spans="3:4">
+      <c r="C52" s="17"/>
+      <c r="D52" s="15"/>
+    </row>
+    <row r="53" s="12" customFormat="1" ht="27" customHeight="1" spans="3:4">
+      <c r="C53" s="17"/>
+      <c r="D53" s="15"/>
+    </row>
+    <row r="54" s="12" customFormat="1" ht="31" customHeight="1" spans="3:4">
+      <c r="C54" s="17"/>
+      <c r="D54" s="15"/>
+    </row>
+    <row r="55" s="12" customFormat="1" ht="36" customHeight="1" spans="3:4">
+      <c r="C55" s="17"/>
+      <c r="D55" s="15"/>
+    </row>
+    <row r="56" s="12" customFormat="1" spans="3:4">
+      <c r="C56" s="17"/>
+      <c r="D56" s="15"/>
+    </row>
+    <row r="57" s="12" customFormat="1" ht="33" customHeight="1" spans="3:4">
+      <c r="C57" s="17"/>
+      <c r="D57" s="15"/>
+    </row>
+    <row r="58" s="12" customFormat="1" ht="32" customHeight="1" spans="3:4">
+      <c r="C58" s="17"/>
+      <c r="D58" s="15"/>
+    </row>
+    <row r="59" s="12" customFormat="1" ht="32" customHeight="1" spans="3:4">
+      <c r="C59" s="17"/>
+      <c r="D59" s="15"/>
+    </row>
+    <row r="60" s="12" customFormat="1" ht="32" customHeight="1" spans="3:4">
+      <c r="C60" s="17"/>
+      <c r="D60" s="15"/>
+    </row>
+    <row r="61" s="12" customFormat="1" ht="33" customHeight="1" spans="3:4">
+      <c r="C61" s="17"/>
+      <c r="D61" s="15"/>
+    </row>
+    <row r="62" s="12" customFormat="1" ht="29" customHeight="1" spans="3:4">
+      <c r="C62" s="17"/>
+      <c r="D62" s="15"/>
+    </row>
+    <row r="63" s="12" customFormat="1" ht="30" customHeight="1" spans="3:4">
+      <c r="C63" s="17"/>
+      <c r="D63" s="15"/>
+    </row>
+    <row r="64" s="12" customFormat="1" ht="29" customHeight="1" spans="3:4">
+      <c r="C64" s="17"/>
+      <c r="D64" s="15"/>
+    </row>
+    <row r="65" s="12" customFormat="1" ht="31" customHeight="1" spans="3:4">
+      <c r="C65" s="17"/>
+      <c r="D65" s="15"/>
+    </row>
+    <row r="66" s="12" customFormat="1" ht="30" customHeight="1" spans="3:4">
+      <c r="C66" s="17"/>
+      <c r="D66" s="15"/>
+    </row>
+    <row r="67" s="12" customFormat="1" ht="33" customHeight="1" spans="3:4">
+      <c r="C67" s="17"/>
+      <c r="D67" s="15"/>
+    </row>
+    <row r="68" s="12" customFormat="1" ht="33" customHeight="1" spans="3:4">
+      <c r="C68" s="17"/>
+      <c r="D68" s="15"/>
+    </row>
+    <row r="69" s="12" customFormat="1" ht="32" customHeight="1" spans="3:4">
+      <c r="C69" s="17"/>
+      <c r="D69" s="15"/>
+    </row>
+    <row r="70" s="12" customFormat="1" ht="32" customHeight="1" spans="3:4">
+      <c r="C70" s="17"/>
+      <c r="D70" s="15"/>
+    </row>
+    <row r="71" s="12" customFormat="1" ht="31" customHeight="1" spans="3:4">
+      <c r="C71" s="17"/>
+      <c r="D71" s="15"/>
+    </row>
+    <row r="72" s="12" customFormat="1" spans="3:4">
+      <c r="C72" s="17"/>
+      <c r="D72" s="15"/>
+    </row>
+    <row r="73" s="12" customFormat="1" spans="3:4">
+      <c r="C73" s="17"/>
+      <c r="D73" s="15"/>
+    </row>
+    <row r="74" s="12" customFormat="1" spans="3:4">
+      <c r="C74" s="17"/>
+      <c r="D74" s="15"/>
+    </row>
+    <row r="75" s="12" customFormat="1" spans="3:4">
+      <c r="C75" s="17"/>
+      <c r="D75" s="15"/>
+    </row>
+    <row r="76" s="12" customFormat="1" spans="3:4">
+      <c r="C76" s="17"/>
+      <c r="D76" s="15"/>
+    </row>
+    <row r="77" s="12" customFormat="1" spans="3:4">
+      <c r="C77" s="17"/>
+      <c r="D77" s="15"/>
+    </row>
+    <row r="78" spans="3:4">
+      <c r="C78" s="17"/>
+      <c r="D78" s="15"/>
+    </row>
+    <row r="79" spans="3:4">
+      <c r="C79" s="17"/>
+      <c r="D79" s="15"/>
+    </row>
+    <row r="80" spans="3:4">
+      <c r="C80" s="17"/>
+      <c r="D80" s="15"/>
+    </row>
+    <row r="81" spans="3:4">
+      <c r="C81" s="17"/>
+      <c r="D81" s="15"/>
+    </row>
+    <row r="82" spans="3:4">
+      <c r="C82" s="17"/>
+      <c r="D82" s="15"/>
+    </row>
+    <row r="83" spans="3:4">
+      <c r="C83" s="17"/>
+      <c r="D83" s="15"/>
+    </row>
+    <row r="84" spans="3:4">
+      <c r="C84" s="17"/>
+      <c r="D84" s="15"/>
+    </row>
+    <row r="85" spans="3:4">
+      <c r="C85" s="17"/>
+      <c r="D85" s="15"/>
+    </row>
+    <row r="86" spans="3:4">
+      <c r="C86" s="17"/>
+      <c r="D86" s="15"/>
+    </row>
+    <row r="87" spans="3:4">
+      <c r="C87" s="17"/>
+      <c r="D87" s="15"/>
+    </row>
+    <row r="88" spans="3:4">
+      <c r="C88" s="17"/>
+      <c r="D88" s="15"/>
+    </row>
+    <row r="89" spans="3:4">
+      <c r="C89" s="17"/>
+      <c r="D89" s="15"/>
+    </row>
+    <row r="90" spans="3:4">
+      <c r="C90" s="17"/>
+      <c r="D90" s="15"/>
+    </row>
+    <row r="91" spans="3:4">
+      <c r="C91" s="17"/>
+      <c r="D91" s="15"/>
+    </row>
+    <row r="92" spans="3:4">
+      <c r="C92" s="17"/>
+      <c r="D92" s="15"/>
+    </row>
+    <row r="93" spans="3:4">
+      <c r="C93" s="17"/>
+      <c r="D93" s="15"/>
+    </row>
+    <row r="94" spans="3:4">
+      <c r="C94" s="17"/>
+      <c r="D94" s="15"/>
+    </row>
+    <row r="95" spans="3:4">
+      <c r="C95" s="17"/>
+      <c r="D95" s="15"/>
+    </row>
+    <row r="96" spans="3:4">
+      <c r="C96" s="17"/>
+      <c r="D96" s="15"/>
+    </row>
+    <row r="97" spans="3:4">
+      <c r="C97" s="17"/>
+      <c r="D97" s="15"/>
+    </row>
+    <row r="98" spans="3:4">
+      <c r="C98" s="17"/>
+      <c r="D98" s="15"/>
+    </row>
+    <row r="99" spans="3:4">
+      <c r="C99" s="17"/>
+      <c r="D99" s="15"/>
+    </row>
+    <row r="100" spans="3:4">
+      <c r="C100" s="17"/>
+      <c r="D100" s="15"/>
+    </row>
+    <row r="101" spans="3:4">
+      <c r="C101" s="17"/>
+      <c r="D101" s="15"/>
+    </row>
+    <row r="102" spans="3:4">
+      <c r="C102" s="17"/>
+      <c r="D102" s="15"/>
+    </row>
+    <row r="103" spans="3:4">
+      <c r="C103" s="17"/>
+      <c r="D103" s="15"/>
+    </row>
+    <row r="104" spans="3:4">
+      <c r="C104" s="17"/>
+      <c r="D104" s="15"/>
+    </row>
+    <row r="105" spans="3:4">
+      <c r="C105" s="17"/>
+      <c r="D105" s="15"/>
+    </row>
+    <row r="106" spans="3:4">
+      <c r="C106" s="17"/>
+      <c r="D106" s="15"/>
+    </row>
+    <row r="107" spans="3:4">
+      <c r="C107" s="17"/>
+      <c r="D107" s="15"/>
+    </row>
+    <row r="108" spans="3:4">
+      <c r="C108" s="17"/>
+      <c r="D108" s="15"/>
+    </row>
+    <row r="109" spans="3:4">
+      <c r="C109" s="17"/>
+      <c r="D109" s="15"/>
+    </row>
+    <row r="110" spans="3:4">
+      <c r="C110" s="17"/>
+      <c r="D110" s="15"/>
+    </row>
+    <row r="111" spans="3:4">
+      <c r="C111" s="17"/>
+      <c r="D111" s="15"/>
+    </row>
+    <row r="112" spans="3:4">
+      <c r="C112" s="17"/>
+      <c r="D112" s="15"/>
+    </row>
+    <row r="113" spans="3:4">
+      <c r="C113" s="17"/>
+      <c r="D113" s="15"/>
+    </row>
+    <row r="114" spans="3:4">
+      <c r="C114" s="17"/>
+      <c r="D114" s="15"/>
+    </row>
+    <row r="115" spans="3:4">
+      <c r="C115" s="17"/>
+      <c r="D115" s="15"/>
+    </row>
+    <row r="116" spans="3:4">
+      <c r="C116" s="17"/>
+      <c r="D116" s="15"/>
+    </row>
+    <row r="117" spans="3:4">
+      <c r="C117" s="17"/>
+      <c r="D117" s="15"/>
+    </row>
+    <row r="118" spans="3:4">
+      <c r="C118" s="17"/>
+      <c r="D118" s="15"/>
+    </row>
+    <row r="119" spans="3:4">
+      <c r="C119" s="17"/>
+      <c r="D119" s="15"/>
+    </row>
+    <row r="120" spans="3:4">
+      <c r="C120" s="17"/>
+      <c r="D120" s="15"/>
+    </row>
+    <row r="121" spans="3:4">
+      <c r="C121" s="17"/>
+      <c r="D121" s="15"/>
+    </row>
+    <row r="122" spans="3:4">
+      <c r="C122" s="17"/>
+      <c r="D122" s="15"/>
+    </row>
+    <row r="123" spans="3:4">
+      <c r="C123" s="17"/>
+      <c r="D123" s="15"/>
+    </row>
+    <row r="124" spans="3:4">
+      <c r="C124" s="17"/>
+      <c r="D124" s="15"/>
+    </row>
+    <row r="125" spans="3:4">
+      <c r="C125" s="17"/>
+      <c r="D125" s="15"/>
+    </row>
+    <row r="126" spans="3:4">
+      <c r="C126" s="18"/>
+      <c r="D126" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>